<commit_message>
Make the tracker's status one tap and self-colouring
She wanted to click that she had written to someone, then whether they replied
or turned her down, and see the state at a glance.

openpyxl cannot emit real checkbox controls, so each status is a dropdown that
colours itself: "Napísala som" turns green, and Výsledok is green for odpísali
or stretnutie, red for odmietli, amber for čakám na odpoveď. Rows she has not
written to yet grey out, so the sheet shows what is outstanding without reading
a word. The same green marks a taken advert and a finished task on the other
sheets.

Prehľad now separates replied, declined and waiting rather than one yes/no, and
counts only rows actually marked as sent. Re-verified against known inputs:
sixteen assertions pass, including a declined reply not counting as an answer.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CRJ8GE4B9NBudRKNSE36EN
</commit_message>
<xml_diff>
--- a/career/Viktoria-hladanie-prace.xlsx
+++ b/career/Viktoria-hladanie-prace.xlsx
@@ -116,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -143,10 +143,79 @@
     <xf numFmtId="1" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <b val="1"/>
+        <color rgb="002E5B1E"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00D6E8C8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <color rgb="008A2F14"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00F3D6CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <color rgb="007A5A12"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FBEBC6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <color rgb="006B6154"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00ECE7E0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -511,1026 +580,1026 @@
   <dimension ref="A1:K55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="38" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Oslovenia — kto, kedy, s čím a čo z toho bolo</t>
+          <t>Oslovenia — komu som napísala a čo z toho bolo</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Vypĺňaš žlté polia. Studené oslovenia najviac jedno za týždeň. Poďakovanie vždy do 24 hodín. Nudge až po štyroch týždňoch ticha a len raz.</t>
+          <t>Ťukni do žltého poľa a vyber zo zoznamu. Bunka sa sama sfarbí: zelená odpísali, červená odmietli, oranžová čakám. Studené oslovenia najviac jedno za týždeň.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>PRÍKLAD:  05.08.2026 | Michal Šajmír | Slovart, výtvarná redakcia | sajmir@slovart.sk | studené | knižné | „Ide to cez odporúčanie alebo cez zaslané portfólio?" | áno | 07.08.2026 | nie | VŠVU, prvá práca v Ikare</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Dátum odoslania</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
+          <t>PRÍKLAD:  áno | 05.08.2026 | Michal Šajmír | Slovart, výtvarná redakcia | sajmir@slovart.sk | studené | knižné | „Ide to cez odporúčanie alebo cez portfólio?" | odpísali | nie | VŠVU</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>Napísala som</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>Dátum</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
         <is>
           <t>Meno</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="D5" s="15" t="inlineStr">
         <is>
           <t>Firma a funkcia</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="E5" s="15" t="inlineStr">
         <is>
           <t>Kontakt</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="F5" s="15" t="inlineStr">
         <is>
           <t>Typ oslovenia</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="G5" s="15" t="inlineStr">
         <is>
           <t>Verzia portfólia</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="H5" s="15" t="inlineStr">
         <is>
           <t>Prosba, ktorú som položila</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>Odpovedal?</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>Dátum odpovede</t>
-        </is>
-      </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>Nudge poslaný?</t>
-        </is>
-      </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>Kde študoval / prvá práca</t>
+      <c r="I5" s="14" t="inlineStr">
+        <is>
+          <t>Výsledok</t>
+        </is>
+      </c>
+      <c r="J5" s="14" t="inlineStr">
+        <is>
+          <t>Nudge</t>
+        </is>
+      </c>
+      <c r="K5" s="15" t="inlineStr">
+        <is>
+          <t>Poznámka</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr"/>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr"/>
+      <c r="B6" s="17" t="inlineStr"/>
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>Michal Šajmír</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="D6" s="18" t="inlineStr">
         <is>
           <t>Slovart — výtvarná redakcia</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="E6" s="18" t="inlineStr">
         <is>
           <t>sajmir@slovart.sk</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="F6" s="18" t="inlineStr">
         <is>
           <t>studené</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="G6" s="18" t="inlineStr">
         <is>
           <t>knižné</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr"/>
-      <c r="H6" s="4" t="inlineStr"/>
-      <c r="I6" s="4" t="inlineStr"/>
-      <c r="J6" s="4" t="inlineStr"/>
-      <c r="K6" s="4" t="inlineStr"/>
+      <c r="H6" s="17" t="inlineStr"/>
+      <c r="I6" s="16" t="inlineStr"/>
+      <c r="J6" s="16" t="inlineStr"/>
+      <c r="K6" s="17" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr"/>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr"/>
+      <c r="B7" s="17" t="inlineStr"/>
+      <c r="C7" s="18" t="inlineStr">
         <is>
           <t>Eva Bubnášová</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="D7" s="18" t="inlineStr">
         <is>
           <t>Spolok sv. Vojtecha, Trnava — šéfredaktorka</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="E7" s="18" t="inlineStr">
         <is>
           <t>sefredaktor@ssv.sk</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="F7" s="18" t="inlineStr">
         <is>
           <t>studené</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="G7" s="18" t="inlineStr">
         <is>
           <t>knižné</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr"/>
-      <c r="H7" s="4" t="inlineStr"/>
-      <c r="I7" s="4" t="inlineStr"/>
-      <c r="J7" s="4" t="inlineStr"/>
-      <c r="K7" s="4" t="inlineStr"/>
+      <c r="H7" s="17" t="inlineStr"/>
+      <c r="I7" s="16" t="inlineStr"/>
+      <c r="J7" s="16" t="inlineStr"/>
+      <c r="K7" s="17" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr"/>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr"/>
+      <c r="B8" s="17" t="inlineStr"/>
+      <c r="C8" s="18" t="inlineStr">
         <is>
           <t>redakcia</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="D8" s="18" t="inlineStr">
         <is>
           <t>Orbis Pictus Istropolitana</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="E8" s="18" t="inlineStr">
         <is>
           <t>redakcia@orbispictus.sk</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="F8" s="18" t="inlineStr">
         <is>
           <t>studené</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="G8" s="18" t="inlineStr">
         <is>
           <t>knižné</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr"/>
-      <c r="H8" s="4" t="inlineStr"/>
-      <c r="I8" s="4" t="inlineStr"/>
-      <c r="J8" s="4" t="inlineStr"/>
-      <c r="K8" s="4" t="inlineStr"/>
+      <c r="H8" s="17" t="inlineStr"/>
+      <c r="I8" s="16" t="inlineStr"/>
+      <c r="J8" s="16" t="inlineStr"/>
+      <c r="K8" s="17" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr"/>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr"/>
+      <c r="B9" s="17" t="inlineStr"/>
+      <c r="C9" s="18" t="inlineStr">
         <is>
           <t>Sandra Friedrichová</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="D9" s="18" t="inlineStr">
         <is>
           <t>Albatros Media — technická redakcia</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="E9" s="18" t="inlineStr">
         <is>
           <t>sandra.friedrichova@albatrosmedia.sk</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="F9" s="18" t="inlineStr">
         <is>
           <t>studené</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="G9" s="18" t="inlineStr">
         <is>
           <t>knižné</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr"/>
-      <c r="H9" s="4" t="inlineStr"/>
-      <c r="I9" s="4" t="inlineStr"/>
-      <c r="J9" s="4" t="inlineStr"/>
-      <c r="K9" s="4" t="inlineStr"/>
+      <c r="H9" s="17" t="inlineStr"/>
+      <c r="I9" s="16" t="inlineStr"/>
+      <c r="J9" s="16" t="inlineStr"/>
+      <c r="K9" s="17" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr"/>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr"/>
+      <c r="B10" s="17" t="inlineStr"/>
+      <c r="C10" s="18" t="inlineStr">
         <is>
           <t>redakcia</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="D10" s="18" t="inlineStr">
         <is>
           <t>Dobrá kniha, Trnava</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="E10" s="18" t="inlineStr">
         <is>
           <t>redakcia@dobrakniha.sk</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="F10" s="18" t="inlineStr">
         <is>
           <t>studené</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="G10" s="18" t="inlineStr">
         <is>
           <t>knižné</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr"/>
-      <c r="H10" s="4" t="inlineStr"/>
-      <c r="I10" s="4" t="inlineStr"/>
-      <c r="J10" s="4" t="inlineStr"/>
-      <c r="K10" s="4" t="inlineStr"/>
+      <c r="H10" s="17" t="inlineStr"/>
+      <c r="I10" s="16" t="inlineStr"/>
+      <c r="J10" s="16" t="inlineStr"/>
+      <c r="K10" s="17" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr"/>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr"/>
+      <c r="B11" s="17" t="inlineStr"/>
+      <c r="C11" s="18" t="inlineStr">
         <is>
           <t>Mária Števková</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="D11" s="18" t="inlineStr">
         <is>
           <t>Buvik — šéfredaktorka</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="E11" s="18" t="inlineStr">
         <is>
           <t>buvik@buvik.sk</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="F11" s="18" t="inlineStr">
         <is>
           <t>studené</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="G11" s="18" t="inlineStr">
         <is>
           <t>knižné</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr"/>
-      <c r="H11" s="4" t="inlineStr"/>
-      <c r="I11" s="4" t="inlineStr"/>
-      <c r="J11" s="4" t="inlineStr"/>
-      <c r="K11" s="4" t="inlineStr"/>
+      <c r="H11" s="17" t="inlineStr"/>
+      <c r="I11" s="16" t="inlineStr"/>
+      <c r="J11" s="16" t="inlineStr"/>
+      <c r="K11" s="17" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr"/>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr"/>
+      <c r="B12" s="17" t="inlineStr"/>
+      <c r="C12" s="18" t="inlineStr">
         <is>
           <t>redakcia</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="D12" s="18" t="inlineStr">
         <is>
           <t>IKAR</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="E12" s="18" t="inlineStr">
         <is>
           <t>redakcia@ikar.sk</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="F12" s="18" t="inlineStr">
         <is>
           <t>studené</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="G12" s="18" t="inlineStr">
         <is>
           <t>knižné</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr"/>
-      <c r="H12" s="4" t="inlineStr"/>
-      <c r="I12" s="4" t="inlineStr"/>
-      <c r="J12" s="4" t="inlineStr"/>
-      <c r="K12" s="4" t="inlineStr"/>
+      <c r="H12" s="17" t="inlineStr"/>
+      <c r="I12" s="16" t="inlineStr"/>
+      <c r="J12" s="16" t="inlineStr"/>
+      <c r="K12" s="17" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr"/>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr"/>
+      <c r="B13" s="17" t="inlineStr"/>
+      <c r="C13" s="18" t="inlineStr">
         <is>
           <t>výstavy</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="D13" s="18" t="inlineStr">
         <is>
           <t>BIBIANA</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="E13" s="18" t="inlineStr">
         <is>
           <t>realizacia@bibiana.sk</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="F13" s="18" t="inlineStr">
         <is>
           <t>studené</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="G13" s="18" t="inlineStr">
         <is>
           <t>knižné</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr"/>
-      <c r="H13" s="4" t="inlineStr"/>
-      <c r="I13" s="4" t="inlineStr"/>
-      <c r="J13" s="4" t="inlineStr"/>
-      <c r="K13" s="4" t="inlineStr"/>
+      <c r="H13" s="17" t="inlineStr"/>
+      <c r="I13" s="16" t="inlineStr"/>
+      <c r="J13" s="16" t="inlineStr"/>
+      <c r="K13" s="17" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr"/>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="A14" s="16" t="inlineStr"/>
+      <c r="B14" s="17" t="inlineStr"/>
+      <c r="C14" s="18" t="inlineStr">
         <is>
           <t>Agáta Petrisková</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="D14" s="18" t="inlineStr">
         <is>
           <t>Slovart — výtvarná redakcia (záloha)</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="E14" s="18" t="inlineStr">
         <is>
           <t>petriskova@slovart.sk</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="F14" s="18" t="inlineStr">
         <is>
           <t>studené</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="G14" s="18" t="inlineStr">
         <is>
           <t>knižné</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr"/>
-      <c r="H14" s="4" t="inlineStr"/>
-      <c r="I14" s="4" t="inlineStr"/>
-      <c r="J14" s="4" t="inlineStr"/>
-      <c r="K14" s="4" t="inlineStr"/>
+      <c r="H14" s="17" t="inlineStr"/>
+      <c r="I14" s="16" t="inlineStr"/>
+      <c r="J14" s="16" t="inlineStr"/>
+      <c r="K14" s="17" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr"/>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr"/>
+      <c r="B15" s="17" t="inlineStr"/>
+      <c r="C15" s="18" t="inlineStr">
         <is>
           <t>personálne oddelenie</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="D15" s="18" t="inlineStr">
         <is>
           <t>Slovenská Grafia — tlačiareň</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="E15" s="18" t="inlineStr">
         <is>
           <t>kariera@grafia.sk</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="F15" s="18" t="inlineStr">
         <is>
           <t>studené</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="G15" s="18" t="inlineStr">
         <is>
           <t>grafické</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr"/>
-      <c r="H15" s="4" t="inlineStr"/>
-      <c r="I15" s="4" t="inlineStr"/>
-      <c r="J15" s="4" t="inlineStr"/>
-      <c r="K15" s="4" t="inlineStr"/>
+      <c r="H15" s="17" t="inlineStr"/>
+      <c r="I15" s="16" t="inlineStr"/>
+      <c r="J15" s="16" t="inlineStr"/>
+      <c r="K15" s="17" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr"/>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr"/>
+      <c r="B16" s="17" t="inlineStr"/>
+      <c r="C16" s="18" t="inlineStr">
         <is>
           <t>[doplň meno]</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="D16" s="18" t="inlineStr">
         <is>
           <t>SOŠ polygrafická — učiteľ</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr"/>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E16" s="18" t="n"/>
+      <c r="F16" s="18" t="inlineStr">
         <is>
           <t>Re-RO</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="G16" s="18" t="inlineStr">
         <is>
           <t>knižné</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr"/>
-      <c r="H16" s="4" t="inlineStr"/>
-      <c r="I16" s="4" t="inlineStr"/>
-      <c r="J16" s="4" t="inlineStr"/>
-      <c r="K16" s="4" t="inlineStr"/>
+      <c r="H16" s="17" t="inlineStr"/>
+      <c r="I16" s="16" t="inlineStr"/>
+      <c r="J16" s="16" t="inlineStr"/>
+      <c r="K16" s="17" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr"/>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr"/>
+      <c r="B17" s="17" t="inlineStr"/>
+      <c r="C17" s="18" t="inlineStr">
         <is>
           <t>[doplň meno]</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="D17" s="18" t="inlineStr">
         <is>
           <t>SOŠ polygrafická — učiteľ</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr"/>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E17" s="18" t="n"/>
+      <c r="F17" s="18" t="inlineStr">
         <is>
           <t>Re-RO</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="G17" s="18" t="inlineStr">
         <is>
           <t>knižné</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr"/>
-      <c r="H17" s="4" t="inlineStr"/>
-      <c r="I17" s="4" t="inlineStr"/>
-      <c r="J17" s="4" t="inlineStr"/>
-      <c r="K17" s="4" t="inlineStr"/>
+      <c r="H17" s="17" t="inlineStr"/>
+      <c r="I17" s="16" t="inlineStr"/>
+      <c r="J17" s="16" t="inlineStr"/>
+      <c r="K17" s="17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr"/>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="A18" s="16" t="inlineStr"/>
+      <c r="B18" s="17" t="inlineStr"/>
+      <c r="C18" s="18" t="inlineStr">
         <is>
           <t>[doplň meno]</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="D18" s="18" t="inlineStr">
         <is>
           <t>PEVŠ — vedúci diplomovky</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr"/>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E18" s="18" t="n"/>
+      <c r="F18" s="18" t="inlineStr">
         <is>
           <t>Re-RO</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="G18" s="18" t="inlineStr">
         <is>
           <t>knižné</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr"/>
-      <c r="H18" s="4" t="inlineStr"/>
-      <c r="I18" s="4" t="inlineStr"/>
-      <c r="J18" s="4" t="inlineStr"/>
-      <c r="K18" s="4" t="inlineStr"/>
+      <c r="H18" s="17" t="inlineStr"/>
+      <c r="I18" s="16" t="inlineStr"/>
+      <c r="J18" s="16" t="inlineStr"/>
+      <c r="K18" s="17" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr"/>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="A19" s="16" t="inlineStr"/>
+      <c r="B19" s="17" t="inlineStr"/>
+      <c r="C19" s="18" t="inlineStr">
         <is>
           <t>[doplň meno]</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="D19" s="18" t="inlineStr">
         <is>
           <t>MOJESIDLO — bývalý kolega</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr"/>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E19" s="18" t="n"/>
+      <c r="F19" s="18" t="inlineStr">
         <is>
           <t>Re-RO</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="G19" s="18" t="inlineStr">
         <is>
           <t>grafické</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr"/>
-      <c r="H19" s="4" t="inlineStr"/>
-      <c r="I19" s="4" t="inlineStr"/>
-      <c r="J19" s="4" t="inlineStr"/>
-      <c r="K19" s="4" t="inlineStr"/>
+      <c r="H19" s="17" t="inlineStr"/>
+      <c r="I19" s="16" t="inlineStr"/>
+      <c r="J19" s="16" t="inlineStr"/>
+      <c r="K19" s="17" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr"/>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="A20" s="16" t="inlineStr"/>
+      <c r="B20" s="17" t="inlineStr"/>
+      <c r="C20" s="18" t="inlineStr">
         <is>
           <t>[doplň meno]</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="D20" s="18" t="inlineStr">
         <is>
           <t>Spolužiak</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr"/>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E20" s="18" t="n"/>
+      <c r="F20" s="18" t="inlineStr">
         <is>
           <t>Re-RO</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="G20" s="18" t="inlineStr">
         <is>
           <t>grafické</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr"/>
-      <c r="H20" s="4" t="inlineStr"/>
-      <c r="I20" s="4" t="inlineStr"/>
-      <c r="J20" s="4" t="inlineStr"/>
-      <c r="K20" s="4" t="inlineStr"/>
+      <c r="H20" s="17" t="inlineStr"/>
+      <c r="I20" s="16" t="inlineStr"/>
+      <c r="J20" s="16" t="inlineStr"/>
+      <c r="K20" s="17" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr"/>
-      <c r="B21" s="4" t="inlineStr"/>
-      <c r="C21" s="4" t="inlineStr"/>
-      <c r="D21" s="4" t="inlineStr"/>
-      <c r="E21" s="4" t="inlineStr"/>
-      <c r="F21" s="4" t="inlineStr"/>
-      <c r="G21" s="4" t="inlineStr"/>
-      <c r="H21" s="4" t="inlineStr"/>
-      <c r="I21" s="4" t="inlineStr"/>
-      <c r="J21" s="4" t="inlineStr"/>
-      <c r="K21" s="4" t="inlineStr"/>
+      <c r="A21" s="16" t="inlineStr"/>
+      <c r="B21" s="17" t="inlineStr"/>
+      <c r="C21" s="17" t="inlineStr"/>
+      <c r="D21" s="17" t="inlineStr"/>
+      <c r="E21" s="17" t="inlineStr"/>
+      <c r="F21" s="17" t="inlineStr"/>
+      <c r="G21" s="17" t="inlineStr"/>
+      <c r="H21" s="17" t="inlineStr"/>
+      <c r="I21" s="16" t="inlineStr"/>
+      <c r="J21" s="16" t="inlineStr"/>
+      <c r="K21" s="17" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr"/>
-      <c r="B22" s="4" t="inlineStr"/>
-      <c r="C22" s="4" t="inlineStr"/>
-      <c r="D22" s="4" t="inlineStr"/>
-      <c r="E22" s="4" t="inlineStr"/>
-      <c r="F22" s="4" t="inlineStr"/>
-      <c r="G22" s="4" t="inlineStr"/>
-      <c r="H22" s="4" t="inlineStr"/>
-      <c r="I22" s="4" t="inlineStr"/>
-      <c r="J22" s="4" t="inlineStr"/>
-      <c r="K22" s="4" t="inlineStr"/>
+      <c r="A22" s="16" t="inlineStr"/>
+      <c r="B22" s="17" t="inlineStr"/>
+      <c r="C22" s="17" t="inlineStr"/>
+      <c r="D22" s="17" t="inlineStr"/>
+      <c r="E22" s="17" t="inlineStr"/>
+      <c r="F22" s="17" t="inlineStr"/>
+      <c r="G22" s="17" t="inlineStr"/>
+      <c r="H22" s="17" t="inlineStr"/>
+      <c r="I22" s="16" t="inlineStr"/>
+      <c r="J22" s="16" t="inlineStr"/>
+      <c r="K22" s="17" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr"/>
-      <c r="B23" s="4" t="inlineStr"/>
-      <c r="C23" s="4" t="inlineStr"/>
-      <c r="D23" s="4" t="inlineStr"/>
-      <c r="E23" s="4" t="inlineStr"/>
-      <c r="F23" s="4" t="inlineStr"/>
-      <c r="G23" s="4" t="inlineStr"/>
-      <c r="H23" s="4" t="inlineStr"/>
-      <c r="I23" s="4" t="inlineStr"/>
-      <c r="J23" s="4" t="inlineStr"/>
-      <c r="K23" s="4" t="inlineStr"/>
+      <c r="A23" s="16" t="inlineStr"/>
+      <c r="B23" s="17" t="inlineStr"/>
+      <c r="C23" s="17" t="inlineStr"/>
+      <c r="D23" s="17" t="inlineStr"/>
+      <c r="E23" s="17" t="inlineStr"/>
+      <c r="F23" s="17" t="inlineStr"/>
+      <c r="G23" s="17" t="inlineStr"/>
+      <c r="H23" s="17" t="inlineStr"/>
+      <c r="I23" s="16" t="inlineStr"/>
+      <c r="J23" s="16" t="inlineStr"/>
+      <c r="K23" s="17" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr"/>
-      <c r="B24" s="4" t="inlineStr"/>
-      <c r="C24" s="4" t="inlineStr"/>
-      <c r="D24" s="4" t="inlineStr"/>
-      <c r="E24" s="4" t="inlineStr"/>
-      <c r="F24" s="4" t="inlineStr"/>
-      <c r="G24" s="4" t="inlineStr"/>
-      <c r="H24" s="4" t="inlineStr"/>
-      <c r="I24" s="4" t="inlineStr"/>
-      <c r="J24" s="4" t="inlineStr"/>
-      <c r="K24" s="4" t="inlineStr"/>
+      <c r="A24" s="16" t="inlineStr"/>
+      <c r="B24" s="17" t="inlineStr"/>
+      <c r="C24" s="17" t="inlineStr"/>
+      <c r="D24" s="17" t="inlineStr"/>
+      <c r="E24" s="17" t="inlineStr"/>
+      <c r="F24" s="17" t="inlineStr"/>
+      <c r="G24" s="17" t="inlineStr"/>
+      <c r="H24" s="17" t="inlineStr"/>
+      <c r="I24" s="16" t="inlineStr"/>
+      <c r="J24" s="16" t="inlineStr"/>
+      <c r="K24" s="17" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr"/>
-      <c r="B25" s="4" t="inlineStr"/>
-      <c r="C25" s="4" t="inlineStr"/>
-      <c r="D25" s="4" t="inlineStr"/>
-      <c r="E25" s="4" t="inlineStr"/>
-      <c r="F25" s="4" t="inlineStr"/>
-      <c r="G25" s="4" t="inlineStr"/>
-      <c r="H25" s="4" t="inlineStr"/>
-      <c r="I25" s="4" t="inlineStr"/>
-      <c r="J25" s="4" t="inlineStr"/>
-      <c r="K25" s="4" t="inlineStr"/>
+      <c r="A25" s="16" t="inlineStr"/>
+      <c r="B25" s="17" t="inlineStr"/>
+      <c r="C25" s="17" t="inlineStr"/>
+      <c r="D25" s="17" t="inlineStr"/>
+      <c r="E25" s="17" t="inlineStr"/>
+      <c r="F25" s="17" t="inlineStr"/>
+      <c r="G25" s="17" t="inlineStr"/>
+      <c r="H25" s="17" t="inlineStr"/>
+      <c r="I25" s="16" t="inlineStr"/>
+      <c r="J25" s="16" t="inlineStr"/>
+      <c r="K25" s="17" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr"/>
-      <c r="B26" s="4" t="inlineStr"/>
-      <c r="C26" s="4" t="inlineStr"/>
-      <c r="D26" s="4" t="inlineStr"/>
-      <c r="E26" s="4" t="inlineStr"/>
-      <c r="F26" s="4" t="inlineStr"/>
-      <c r="G26" s="4" t="inlineStr"/>
-      <c r="H26" s="4" t="inlineStr"/>
-      <c r="I26" s="4" t="inlineStr"/>
-      <c r="J26" s="4" t="inlineStr"/>
-      <c r="K26" s="4" t="inlineStr"/>
+      <c r="A26" s="16" t="inlineStr"/>
+      <c r="B26" s="17" t="inlineStr"/>
+      <c r="C26" s="17" t="inlineStr"/>
+      <c r="D26" s="17" t="inlineStr"/>
+      <c r="E26" s="17" t="inlineStr"/>
+      <c r="F26" s="17" t="inlineStr"/>
+      <c r="G26" s="17" t="inlineStr"/>
+      <c r="H26" s="17" t="inlineStr"/>
+      <c r="I26" s="16" t="inlineStr"/>
+      <c r="J26" s="16" t="inlineStr"/>
+      <c r="K26" s="17" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr"/>
-      <c r="B27" s="4" t="inlineStr"/>
-      <c r="C27" s="4" t="inlineStr"/>
-      <c r="D27" s="4" t="inlineStr"/>
-      <c r="E27" s="4" t="inlineStr"/>
-      <c r="F27" s="4" t="inlineStr"/>
-      <c r="G27" s="4" t="inlineStr"/>
-      <c r="H27" s="4" t="inlineStr"/>
-      <c r="I27" s="4" t="inlineStr"/>
-      <c r="J27" s="4" t="inlineStr"/>
-      <c r="K27" s="4" t="inlineStr"/>
+      <c r="A27" s="16" t="inlineStr"/>
+      <c r="B27" s="17" t="inlineStr"/>
+      <c r="C27" s="17" t="inlineStr"/>
+      <c r="D27" s="17" t="inlineStr"/>
+      <c r="E27" s="17" t="inlineStr"/>
+      <c r="F27" s="17" t="inlineStr"/>
+      <c r="G27" s="17" t="inlineStr"/>
+      <c r="H27" s="17" t="inlineStr"/>
+      <c r="I27" s="16" t="inlineStr"/>
+      <c r="J27" s="16" t="inlineStr"/>
+      <c r="K27" s="17" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr"/>
-      <c r="B28" s="4" t="inlineStr"/>
-      <c r="C28" s="4" t="inlineStr"/>
-      <c r="D28" s="4" t="inlineStr"/>
-      <c r="E28" s="4" t="inlineStr"/>
-      <c r="F28" s="4" t="inlineStr"/>
-      <c r="G28" s="4" t="inlineStr"/>
-      <c r="H28" s="4" t="inlineStr"/>
-      <c r="I28" s="4" t="inlineStr"/>
-      <c r="J28" s="4" t="inlineStr"/>
-      <c r="K28" s="4" t="inlineStr"/>
+      <c r="A28" s="16" t="inlineStr"/>
+      <c r="B28" s="17" t="inlineStr"/>
+      <c r="C28" s="17" t="inlineStr"/>
+      <c r="D28" s="17" t="inlineStr"/>
+      <c r="E28" s="17" t="inlineStr"/>
+      <c r="F28" s="17" t="inlineStr"/>
+      <c r="G28" s="17" t="inlineStr"/>
+      <c r="H28" s="17" t="inlineStr"/>
+      <c r="I28" s="16" t="inlineStr"/>
+      <c r="J28" s="16" t="inlineStr"/>
+      <c r="K28" s="17" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr"/>
-      <c r="B29" s="4" t="inlineStr"/>
-      <c r="C29" s="4" t="inlineStr"/>
-      <c r="D29" s="4" t="inlineStr"/>
-      <c r="E29" s="4" t="inlineStr"/>
-      <c r="F29" s="4" t="inlineStr"/>
-      <c r="G29" s="4" t="inlineStr"/>
-      <c r="H29" s="4" t="inlineStr"/>
-      <c r="I29" s="4" t="inlineStr"/>
-      <c r="J29" s="4" t="inlineStr"/>
-      <c r="K29" s="4" t="inlineStr"/>
+      <c r="A29" s="16" t="inlineStr"/>
+      <c r="B29" s="17" t="inlineStr"/>
+      <c r="C29" s="17" t="inlineStr"/>
+      <c r="D29" s="17" t="inlineStr"/>
+      <c r="E29" s="17" t="inlineStr"/>
+      <c r="F29" s="17" t="inlineStr"/>
+      <c r="G29" s="17" t="inlineStr"/>
+      <c r="H29" s="17" t="inlineStr"/>
+      <c r="I29" s="16" t="inlineStr"/>
+      <c r="J29" s="16" t="inlineStr"/>
+      <c r="K29" s="17" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr"/>
-      <c r="B30" s="4" t="inlineStr"/>
-      <c r="C30" s="4" t="inlineStr"/>
-      <c r="D30" s="4" t="inlineStr"/>
-      <c r="E30" s="4" t="inlineStr"/>
-      <c r="F30" s="4" t="inlineStr"/>
-      <c r="G30" s="4" t="inlineStr"/>
-      <c r="H30" s="4" t="inlineStr"/>
-      <c r="I30" s="4" t="inlineStr"/>
-      <c r="J30" s="4" t="inlineStr"/>
-      <c r="K30" s="4" t="inlineStr"/>
+      <c r="A30" s="16" t="inlineStr"/>
+      <c r="B30" s="17" t="inlineStr"/>
+      <c r="C30" s="17" t="inlineStr"/>
+      <c r="D30" s="17" t="inlineStr"/>
+      <c r="E30" s="17" t="inlineStr"/>
+      <c r="F30" s="17" t="inlineStr"/>
+      <c r="G30" s="17" t="inlineStr"/>
+      <c r="H30" s="17" t="inlineStr"/>
+      <c r="I30" s="16" t="inlineStr"/>
+      <c r="J30" s="16" t="inlineStr"/>
+      <c r="K30" s="17" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr"/>
-      <c r="B31" s="4" t="inlineStr"/>
-      <c r="C31" s="4" t="inlineStr"/>
-      <c r="D31" s="4" t="inlineStr"/>
-      <c r="E31" s="4" t="inlineStr"/>
-      <c r="F31" s="4" t="inlineStr"/>
-      <c r="G31" s="4" t="inlineStr"/>
-      <c r="H31" s="4" t="inlineStr"/>
-      <c r="I31" s="4" t="inlineStr"/>
-      <c r="J31" s="4" t="inlineStr"/>
-      <c r="K31" s="4" t="inlineStr"/>
+      <c r="A31" s="16" t="inlineStr"/>
+      <c r="B31" s="17" t="inlineStr"/>
+      <c r="C31" s="17" t="inlineStr"/>
+      <c r="D31" s="17" t="inlineStr"/>
+      <c r="E31" s="17" t="inlineStr"/>
+      <c r="F31" s="17" t="inlineStr"/>
+      <c r="G31" s="17" t="inlineStr"/>
+      <c r="H31" s="17" t="inlineStr"/>
+      <c r="I31" s="16" t="inlineStr"/>
+      <c r="J31" s="16" t="inlineStr"/>
+      <c r="K31" s="17" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr"/>
-      <c r="B32" s="4" t="inlineStr"/>
-      <c r="C32" s="4" t="inlineStr"/>
-      <c r="D32" s="4" t="inlineStr"/>
-      <c r="E32" s="4" t="inlineStr"/>
-      <c r="F32" s="4" t="inlineStr"/>
-      <c r="G32" s="4" t="inlineStr"/>
-      <c r="H32" s="4" t="inlineStr"/>
-      <c r="I32" s="4" t="inlineStr"/>
-      <c r="J32" s="4" t="inlineStr"/>
-      <c r="K32" s="4" t="inlineStr"/>
+      <c r="A32" s="16" t="inlineStr"/>
+      <c r="B32" s="17" t="inlineStr"/>
+      <c r="C32" s="17" t="inlineStr"/>
+      <c r="D32" s="17" t="inlineStr"/>
+      <c r="E32" s="17" t="inlineStr"/>
+      <c r="F32" s="17" t="inlineStr"/>
+      <c r="G32" s="17" t="inlineStr"/>
+      <c r="H32" s="17" t="inlineStr"/>
+      <c r="I32" s="16" t="inlineStr"/>
+      <c r="J32" s="16" t="inlineStr"/>
+      <c r="K32" s="17" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="inlineStr"/>
-      <c r="B33" s="4" t="inlineStr"/>
-      <c r="C33" s="4" t="inlineStr"/>
-      <c r="D33" s="4" t="inlineStr"/>
-      <c r="E33" s="4" t="inlineStr"/>
-      <c r="F33" s="4" t="inlineStr"/>
-      <c r="G33" s="4" t="inlineStr"/>
-      <c r="H33" s="4" t="inlineStr"/>
-      <c r="I33" s="4" t="inlineStr"/>
-      <c r="J33" s="4" t="inlineStr"/>
-      <c r="K33" s="4" t="inlineStr"/>
+      <c r="A33" s="16" t="inlineStr"/>
+      <c r="B33" s="17" t="inlineStr"/>
+      <c r="C33" s="17" t="inlineStr"/>
+      <c r="D33" s="17" t="inlineStr"/>
+      <c r="E33" s="17" t="inlineStr"/>
+      <c r="F33" s="17" t="inlineStr"/>
+      <c r="G33" s="17" t="inlineStr"/>
+      <c r="H33" s="17" t="inlineStr"/>
+      <c r="I33" s="16" t="inlineStr"/>
+      <c r="J33" s="16" t="inlineStr"/>
+      <c r="K33" s="17" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="inlineStr"/>
-      <c r="B34" s="4" t="inlineStr"/>
-      <c r="C34" s="4" t="inlineStr"/>
-      <c r="D34" s="4" t="inlineStr"/>
-      <c r="E34" s="4" t="inlineStr"/>
-      <c r="F34" s="4" t="inlineStr"/>
-      <c r="G34" s="4" t="inlineStr"/>
-      <c r="H34" s="4" t="inlineStr"/>
-      <c r="I34" s="4" t="inlineStr"/>
-      <c r="J34" s="4" t="inlineStr"/>
-      <c r="K34" s="4" t="inlineStr"/>
+      <c r="A34" s="16" t="inlineStr"/>
+      <c r="B34" s="17" t="inlineStr"/>
+      <c r="C34" s="17" t="inlineStr"/>
+      <c r="D34" s="17" t="inlineStr"/>
+      <c r="E34" s="17" t="inlineStr"/>
+      <c r="F34" s="17" t="inlineStr"/>
+      <c r="G34" s="17" t="inlineStr"/>
+      <c r="H34" s="17" t="inlineStr"/>
+      <c r="I34" s="16" t="inlineStr"/>
+      <c r="J34" s="16" t="inlineStr"/>
+      <c r="K34" s="17" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="inlineStr"/>
-      <c r="B35" s="4" t="inlineStr"/>
-      <c r="C35" s="4" t="inlineStr"/>
-      <c r="D35" s="4" t="inlineStr"/>
-      <c r="E35" s="4" t="inlineStr"/>
-      <c r="F35" s="4" t="inlineStr"/>
-      <c r="G35" s="4" t="inlineStr"/>
-      <c r="H35" s="4" t="inlineStr"/>
-      <c r="I35" s="4" t="inlineStr"/>
-      <c r="J35" s="4" t="inlineStr"/>
-      <c r="K35" s="4" t="inlineStr"/>
+      <c r="A35" s="16" t="inlineStr"/>
+      <c r="B35" s="17" t="inlineStr"/>
+      <c r="C35" s="17" t="inlineStr"/>
+      <c r="D35" s="17" t="inlineStr"/>
+      <c r="E35" s="17" t="inlineStr"/>
+      <c r="F35" s="17" t="inlineStr"/>
+      <c r="G35" s="17" t="inlineStr"/>
+      <c r="H35" s="17" t="inlineStr"/>
+      <c r="I35" s="16" t="inlineStr"/>
+      <c r="J35" s="16" t="inlineStr"/>
+      <c r="K35" s="17" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="inlineStr"/>
-      <c r="B36" s="4" t="inlineStr"/>
-      <c r="C36" s="4" t="inlineStr"/>
-      <c r="D36" s="4" t="inlineStr"/>
-      <c r="E36" s="4" t="inlineStr"/>
-      <c r="F36" s="4" t="inlineStr"/>
-      <c r="G36" s="4" t="inlineStr"/>
-      <c r="H36" s="4" t="inlineStr"/>
-      <c r="I36" s="4" t="inlineStr"/>
-      <c r="J36" s="4" t="inlineStr"/>
-      <c r="K36" s="4" t="inlineStr"/>
+      <c r="A36" s="16" t="inlineStr"/>
+      <c r="B36" s="17" t="inlineStr"/>
+      <c r="C36" s="17" t="inlineStr"/>
+      <c r="D36" s="17" t="inlineStr"/>
+      <c r="E36" s="17" t="inlineStr"/>
+      <c r="F36" s="17" t="inlineStr"/>
+      <c r="G36" s="17" t="inlineStr"/>
+      <c r="H36" s="17" t="inlineStr"/>
+      <c r="I36" s="16" t="inlineStr"/>
+      <c r="J36" s="16" t="inlineStr"/>
+      <c r="K36" s="17" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="inlineStr"/>
-      <c r="B37" s="4" t="inlineStr"/>
-      <c r="C37" s="4" t="inlineStr"/>
-      <c r="D37" s="4" t="inlineStr"/>
-      <c r="E37" s="4" t="inlineStr"/>
-      <c r="F37" s="4" t="inlineStr"/>
-      <c r="G37" s="4" t="inlineStr"/>
-      <c r="H37" s="4" t="inlineStr"/>
-      <c r="I37" s="4" t="inlineStr"/>
-      <c r="J37" s="4" t="inlineStr"/>
-      <c r="K37" s="4" t="inlineStr"/>
+      <c r="A37" s="16" t="inlineStr"/>
+      <c r="B37" s="17" t="inlineStr"/>
+      <c r="C37" s="17" t="inlineStr"/>
+      <c r="D37" s="17" t="inlineStr"/>
+      <c r="E37" s="17" t="inlineStr"/>
+      <c r="F37" s="17" t="inlineStr"/>
+      <c r="G37" s="17" t="inlineStr"/>
+      <c r="H37" s="17" t="inlineStr"/>
+      <c r="I37" s="16" t="inlineStr"/>
+      <c r="J37" s="16" t="inlineStr"/>
+      <c r="K37" s="17" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="inlineStr"/>
-      <c r="B38" s="4" t="inlineStr"/>
-      <c r="C38" s="4" t="inlineStr"/>
-      <c r="D38" s="4" t="inlineStr"/>
-      <c r="E38" s="4" t="inlineStr"/>
-      <c r="F38" s="4" t="inlineStr"/>
-      <c r="G38" s="4" t="inlineStr"/>
-      <c r="H38" s="4" t="inlineStr"/>
-      <c r="I38" s="4" t="inlineStr"/>
-      <c r="J38" s="4" t="inlineStr"/>
-      <c r="K38" s="4" t="inlineStr"/>
+      <c r="A38" s="16" t="inlineStr"/>
+      <c r="B38" s="17" t="inlineStr"/>
+      <c r="C38" s="17" t="inlineStr"/>
+      <c r="D38" s="17" t="inlineStr"/>
+      <c r="E38" s="17" t="inlineStr"/>
+      <c r="F38" s="17" t="inlineStr"/>
+      <c r="G38" s="17" t="inlineStr"/>
+      <c r="H38" s="17" t="inlineStr"/>
+      <c r="I38" s="16" t="inlineStr"/>
+      <c r="J38" s="16" t="inlineStr"/>
+      <c r="K38" s="17" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="inlineStr"/>
-      <c r="B39" s="4" t="inlineStr"/>
-      <c r="C39" s="4" t="inlineStr"/>
-      <c r="D39" s="4" t="inlineStr"/>
-      <c r="E39" s="4" t="inlineStr"/>
-      <c r="F39" s="4" t="inlineStr"/>
-      <c r="G39" s="4" t="inlineStr"/>
-      <c r="H39" s="4" t="inlineStr"/>
-      <c r="I39" s="4" t="inlineStr"/>
-      <c r="J39" s="4" t="inlineStr"/>
-      <c r="K39" s="4" t="inlineStr"/>
+      <c r="A39" s="16" t="inlineStr"/>
+      <c r="B39" s="17" t="inlineStr"/>
+      <c r="C39" s="17" t="inlineStr"/>
+      <c r="D39" s="17" t="inlineStr"/>
+      <c r="E39" s="17" t="inlineStr"/>
+      <c r="F39" s="17" t="inlineStr"/>
+      <c r="G39" s="17" t="inlineStr"/>
+      <c r="H39" s="17" t="inlineStr"/>
+      <c r="I39" s="16" t="inlineStr"/>
+      <c r="J39" s="16" t="inlineStr"/>
+      <c r="K39" s="17" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="4" t="inlineStr"/>
-      <c r="B40" s="4" t="inlineStr"/>
-      <c r="C40" s="4" t="inlineStr"/>
-      <c r="D40" s="4" t="inlineStr"/>
-      <c r="E40" s="4" t="inlineStr"/>
-      <c r="F40" s="4" t="inlineStr"/>
-      <c r="G40" s="4" t="inlineStr"/>
-      <c r="H40" s="4" t="inlineStr"/>
-      <c r="I40" s="4" t="inlineStr"/>
-      <c r="J40" s="4" t="inlineStr"/>
-      <c r="K40" s="4" t="inlineStr"/>
+      <c r="A40" s="16" t="inlineStr"/>
+      <c r="B40" s="17" t="inlineStr"/>
+      <c r="C40" s="17" t="inlineStr"/>
+      <c r="D40" s="17" t="inlineStr"/>
+      <c r="E40" s="17" t="inlineStr"/>
+      <c r="F40" s="17" t="inlineStr"/>
+      <c r="G40" s="17" t="inlineStr"/>
+      <c r="H40" s="17" t="inlineStr"/>
+      <c r="I40" s="16" t="inlineStr"/>
+      <c r="J40" s="16" t="inlineStr"/>
+      <c r="K40" s="17" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="4" t="inlineStr"/>
-      <c r="B41" s="4" t="inlineStr"/>
-      <c r="C41" s="4" t="inlineStr"/>
-      <c r="D41" s="4" t="inlineStr"/>
-      <c r="E41" s="4" t="inlineStr"/>
-      <c r="F41" s="4" t="inlineStr"/>
-      <c r="G41" s="4" t="inlineStr"/>
-      <c r="H41" s="4" t="inlineStr"/>
-      <c r="I41" s="4" t="inlineStr"/>
-      <c r="J41" s="4" t="inlineStr"/>
-      <c r="K41" s="4" t="inlineStr"/>
+      <c r="A41" s="16" t="inlineStr"/>
+      <c r="B41" s="17" t="inlineStr"/>
+      <c r="C41" s="17" t="inlineStr"/>
+      <c r="D41" s="17" t="inlineStr"/>
+      <c r="E41" s="17" t="inlineStr"/>
+      <c r="F41" s="17" t="inlineStr"/>
+      <c r="G41" s="17" t="inlineStr"/>
+      <c r="H41" s="17" t="inlineStr"/>
+      <c r="I41" s="16" t="inlineStr"/>
+      <c r="J41" s="16" t="inlineStr"/>
+      <c r="K41" s="17" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="4" t="inlineStr"/>
-      <c r="B42" s="4" t="inlineStr"/>
-      <c r="C42" s="4" t="inlineStr"/>
-      <c r="D42" s="4" t="inlineStr"/>
-      <c r="E42" s="4" t="inlineStr"/>
-      <c r="F42" s="4" t="inlineStr"/>
-      <c r="G42" s="4" t="inlineStr"/>
-      <c r="H42" s="4" t="inlineStr"/>
-      <c r="I42" s="4" t="inlineStr"/>
-      <c r="J42" s="4" t="inlineStr"/>
-      <c r="K42" s="4" t="inlineStr"/>
+      <c r="A42" s="16" t="inlineStr"/>
+      <c r="B42" s="17" t="inlineStr"/>
+      <c r="C42" s="17" t="inlineStr"/>
+      <c r="D42" s="17" t="inlineStr"/>
+      <c r="E42" s="17" t="inlineStr"/>
+      <c r="F42" s="17" t="inlineStr"/>
+      <c r="G42" s="17" t="inlineStr"/>
+      <c r="H42" s="17" t="inlineStr"/>
+      <c r="I42" s="16" t="inlineStr"/>
+      <c r="J42" s="16" t="inlineStr"/>
+      <c r="K42" s="17" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="inlineStr"/>
-      <c r="B43" s="4" t="inlineStr"/>
-      <c r="C43" s="4" t="inlineStr"/>
-      <c r="D43" s="4" t="inlineStr"/>
-      <c r="E43" s="4" t="inlineStr"/>
-      <c r="F43" s="4" t="inlineStr"/>
-      <c r="G43" s="4" t="inlineStr"/>
-      <c r="H43" s="4" t="inlineStr"/>
-      <c r="I43" s="4" t="inlineStr"/>
-      <c r="J43" s="4" t="inlineStr"/>
-      <c r="K43" s="4" t="inlineStr"/>
+      <c r="A43" s="16" t="inlineStr"/>
+      <c r="B43" s="17" t="inlineStr"/>
+      <c r="C43" s="17" t="inlineStr"/>
+      <c r="D43" s="17" t="inlineStr"/>
+      <c r="E43" s="17" t="inlineStr"/>
+      <c r="F43" s="17" t="inlineStr"/>
+      <c r="G43" s="17" t="inlineStr"/>
+      <c r="H43" s="17" t="inlineStr"/>
+      <c r="I43" s="16" t="inlineStr"/>
+      <c r="J43" s="16" t="inlineStr"/>
+      <c r="K43" s="17" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="4" t="inlineStr"/>
-      <c r="B44" s="4" t="inlineStr"/>
-      <c r="C44" s="4" t="inlineStr"/>
-      <c r="D44" s="4" t="inlineStr"/>
-      <c r="E44" s="4" t="inlineStr"/>
-      <c r="F44" s="4" t="inlineStr"/>
-      <c r="G44" s="4" t="inlineStr"/>
-      <c r="H44" s="4" t="inlineStr"/>
-      <c r="I44" s="4" t="inlineStr"/>
-      <c r="J44" s="4" t="inlineStr"/>
-      <c r="K44" s="4" t="inlineStr"/>
+      <c r="A44" s="16" t="inlineStr"/>
+      <c r="B44" s="17" t="inlineStr"/>
+      <c r="C44" s="17" t="inlineStr"/>
+      <c r="D44" s="17" t="inlineStr"/>
+      <c r="E44" s="17" t="inlineStr"/>
+      <c r="F44" s="17" t="inlineStr"/>
+      <c r="G44" s="17" t="inlineStr"/>
+      <c r="H44" s="17" t="inlineStr"/>
+      <c r="I44" s="16" t="inlineStr"/>
+      <c r="J44" s="16" t="inlineStr"/>
+      <c r="K44" s="17" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="inlineStr"/>
-      <c r="B45" s="4" t="inlineStr"/>
-      <c r="C45" s="4" t="inlineStr"/>
-      <c r="D45" s="4" t="inlineStr"/>
-      <c r="E45" s="4" t="inlineStr"/>
-      <c r="F45" s="4" t="inlineStr"/>
-      <c r="G45" s="4" t="inlineStr"/>
-      <c r="H45" s="4" t="inlineStr"/>
-      <c r="I45" s="4" t="inlineStr"/>
-      <c r="J45" s="4" t="inlineStr"/>
-      <c r="K45" s="4" t="inlineStr"/>
+      <c r="A45" s="16" t="inlineStr"/>
+      <c r="B45" s="17" t="inlineStr"/>
+      <c r="C45" s="17" t="inlineStr"/>
+      <c r="D45" s="17" t="inlineStr"/>
+      <c r="E45" s="17" t="inlineStr"/>
+      <c r="F45" s="17" t="inlineStr"/>
+      <c r="G45" s="17" t="inlineStr"/>
+      <c r="H45" s="17" t="inlineStr"/>
+      <c r="I45" s="16" t="inlineStr"/>
+      <c r="J45" s="16" t="inlineStr"/>
+      <c r="K45" s="17" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="4" t="inlineStr"/>
-      <c r="B46" s="4" t="inlineStr"/>
-      <c r="C46" s="4" t="inlineStr"/>
-      <c r="D46" s="4" t="inlineStr"/>
-      <c r="E46" s="4" t="inlineStr"/>
-      <c r="F46" s="4" t="inlineStr"/>
-      <c r="G46" s="4" t="inlineStr"/>
-      <c r="H46" s="4" t="inlineStr"/>
-      <c r="I46" s="4" t="inlineStr"/>
-      <c r="J46" s="4" t="inlineStr"/>
-      <c r="K46" s="4" t="inlineStr"/>
+      <c r="A46" s="16" t="inlineStr"/>
+      <c r="B46" s="17" t="inlineStr"/>
+      <c r="C46" s="17" t="inlineStr"/>
+      <c r="D46" s="17" t="inlineStr"/>
+      <c r="E46" s="17" t="inlineStr"/>
+      <c r="F46" s="17" t="inlineStr"/>
+      <c r="G46" s="17" t="inlineStr"/>
+      <c r="H46" s="17" t="inlineStr"/>
+      <c r="I46" s="16" t="inlineStr"/>
+      <c r="J46" s="16" t="inlineStr"/>
+      <c r="K46" s="17" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="4" t="inlineStr"/>
-      <c r="B47" s="4" t="inlineStr"/>
-      <c r="C47" s="4" t="inlineStr"/>
-      <c r="D47" s="4" t="inlineStr"/>
-      <c r="E47" s="4" t="inlineStr"/>
-      <c r="F47" s="4" t="inlineStr"/>
-      <c r="G47" s="4" t="inlineStr"/>
-      <c r="H47" s="4" t="inlineStr"/>
-      <c r="I47" s="4" t="inlineStr"/>
-      <c r="J47" s="4" t="inlineStr"/>
-      <c r="K47" s="4" t="inlineStr"/>
+      <c r="A47" s="16" t="inlineStr"/>
+      <c r="B47" s="17" t="inlineStr"/>
+      <c r="C47" s="17" t="inlineStr"/>
+      <c r="D47" s="17" t="inlineStr"/>
+      <c r="E47" s="17" t="inlineStr"/>
+      <c r="F47" s="17" t="inlineStr"/>
+      <c r="G47" s="17" t="inlineStr"/>
+      <c r="H47" s="17" t="inlineStr"/>
+      <c r="I47" s="16" t="inlineStr"/>
+      <c r="J47" s="16" t="inlineStr"/>
+      <c r="K47" s="17" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="4" t="inlineStr"/>
-      <c r="B48" s="4" t="inlineStr"/>
-      <c r="C48" s="4" t="inlineStr"/>
-      <c r="D48" s="4" t="inlineStr"/>
-      <c r="E48" s="4" t="inlineStr"/>
-      <c r="F48" s="4" t="inlineStr"/>
-      <c r="G48" s="4" t="inlineStr"/>
-      <c r="H48" s="4" t="inlineStr"/>
-      <c r="I48" s="4" t="inlineStr"/>
-      <c r="J48" s="4" t="inlineStr"/>
-      <c r="K48" s="4" t="inlineStr"/>
+      <c r="A48" s="16" t="inlineStr"/>
+      <c r="B48" s="17" t="inlineStr"/>
+      <c r="C48" s="17" t="inlineStr"/>
+      <c r="D48" s="17" t="inlineStr"/>
+      <c r="E48" s="17" t="inlineStr"/>
+      <c r="F48" s="17" t="inlineStr"/>
+      <c r="G48" s="17" t="inlineStr"/>
+      <c r="H48" s="17" t="inlineStr"/>
+      <c r="I48" s="16" t="inlineStr"/>
+      <c r="J48" s="16" t="inlineStr"/>
+      <c r="K48" s="17" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="4" t="inlineStr"/>
-      <c r="B49" s="4" t="inlineStr"/>
-      <c r="C49" s="4" t="inlineStr"/>
-      <c r="D49" s="4" t="inlineStr"/>
-      <c r="E49" s="4" t="inlineStr"/>
-      <c r="F49" s="4" t="inlineStr"/>
-      <c r="G49" s="4" t="inlineStr"/>
-      <c r="H49" s="4" t="inlineStr"/>
-      <c r="I49" s="4" t="inlineStr"/>
-      <c r="J49" s="4" t="inlineStr"/>
-      <c r="K49" s="4" t="inlineStr"/>
+      <c r="A49" s="16" t="inlineStr"/>
+      <c r="B49" s="17" t="inlineStr"/>
+      <c r="C49" s="17" t="inlineStr"/>
+      <c r="D49" s="17" t="inlineStr"/>
+      <c r="E49" s="17" t="inlineStr"/>
+      <c r="F49" s="17" t="inlineStr"/>
+      <c r="G49" s="17" t="inlineStr"/>
+      <c r="H49" s="17" t="inlineStr"/>
+      <c r="I49" s="16" t="inlineStr"/>
+      <c r="J49" s="16" t="inlineStr"/>
+      <c r="K49" s="17" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="4" t="inlineStr"/>
-      <c r="B50" s="4" t="inlineStr"/>
-      <c r="C50" s="4" t="inlineStr"/>
-      <c r="D50" s="4" t="inlineStr"/>
-      <c r="E50" s="4" t="inlineStr"/>
-      <c r="F50" s="4" t="inlineStr"/>
-      <c r="G50" s="4" t="inlineStr"/>
-      <c r="H50" s="4" t="inlineStr"/>
-      <c r="I50" s="4" t="inlineStr"/>
-      <c r="J50" s="4" t="inlineStr"/>
-      <c r="K50" s="4" t="inlineStr"/>
+      <c r="A50" s="16" t="inlineStr"/>
+      <c r="B50" s="17" t="inlineStr"/>
+      <c r="C50" s="17" t="inlineStr"/>
+      <c r="D50" s="17" t="inlineStr"/>
+      <c r="E50" s="17" t="inlineStr"/>
+      <c r="F50" s="17" t="inlineStr"/>
+      <c r="G50" s="17" t="inlineStr"/>
+      <c r="H50" s="17" t="inlineStr"/>
+      <c r="I50" s="16" t="inlineStr"/>
+      <c r="J50" s="16" t="inlineStr"/>
+      <c r="K50" s="17" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="4" t="inlineStr"/>
-      <c r="B51" s="4" t="inlineStr"/>
-      <c r="C51" s="4" t="inlineStr"/>
-      <c r="D51" s="4" t="inlineStr"/>
-      <c r="E51" s="4" t="inlineStr"/>
-      <c r="F51" s="4" t="inlineStr"/>
-      <c r="G51" s="4" t="inlineStr"/>
-      <c r="H51" s="4" t="inlineStr"/>
-      <c r="I51" s="4" t="inlineStr"/>
-      <c r="J51" s="4" t="inlineStr"/>
-      <c r="K51" s="4" t="inlineStr"/>
+      <c r="A51" s="16" t="inlineStr"/>
+      <c r="B51" s="17" t="inlineStr"/>
+      <c r="C51" s="17" t="inlineStr"/>
+      <c r="D51" s="17" t="inlineStr"/>
+      <c r="E51" s="17" t="inlineStr"/>
+      <c r="F51" s="17" t="inlineStr"/>
+      <c r="G51" s="17" t="inlineStr"/>
+      <c r="H51" s="17" t="inlineStr"/>
+      <c r="I51" s="16" t="inlineStr"/>
+      <c r="J51" s="16" t="inlineStr"/>
+      <c r="K51" s="17" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="4" t="inlineStr"/>
-      <c r="B52" s="4" t="inlineStr"/>
-      <c r="C52" s="4" t="inlineStr"/>
-      <c r="D52" s="4" t="inlineStr"/>
-      <c r="E52" s="4" t="inlineStr"/>
-      <c r="F52" s="4" t="inlineStr"/>
-      <c r="G52" s="4" t="inlineStr"/>
-      <c r="H52" s="4" t="inlineStr"/>
-      <c r="I52" s="4" t="inlineStr"/>
-      <c r="J52" s="4" t="inlineStr"/>
-      <c r="K52" s="4" t="inlineStr"/>
+      <c r="A52" s="16" t="inlineStr"/>
+      <c r="B52" s="17" t="inlineStr"/>
+      <c r="C52" s="17" t="inlineStr"/>
+      <c r="D52" s="17" t="inlineStr"/>
+      <c r="E52" s="17" t="inlineStr"/>
+      <c r="F52" s="17" t="inlineStr"/>
+      <c r="G52" s="17" t="inlineStr"/>
+      <c r="H52" s="17" t="inlineStr"/>
+      <c r="I52" s="16" t="inlineStr"/>
+      <c r="J52" s="16" t="inlineStr"/>
+      <c r="K52" s="17" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="4" t="inlineStr"/>
-      <c r="B53" s="4" t="inlineStr"/>
-      <c r="C53" s="4" t="inlineStr"/>
-      <c r="D53" s="4" t="inlineStr"/>
-      <c r="E53" s="4" t="inlineStr"/>
-      <c r="F53" s="4" t="inlineStr"/>
-      <c r="G53" s="4" t="inlineStr"/>
-      <c r="H53" s="4" t="inlineStr"/>
-      <c r="I53" s="4" t="inlineStr"/>
-      <c r="J53" s="4" t="inlineStr"/>
-      <c r="K53" s="4" t="inlineStr"/>
+      <c r="A53" s="16" t="inlineStr"/>
+      <c r="B53" s="17" t="inlineStr"/>
+      <c r="C53" s="17" t="inlineStr"/>
+      <c r="D53" s="17" t="inlineStr"/>
+      <c r="E53" s="17" t="inlineStr"/>
+      <c r="F53" s="17" t="inlineStr"/>
+      <c r="G53" s="17" t="inlineStr"/>
+      <c r="H53" s="17" t="inlineStr"/>
+      <c r="I53" s="16" t="inlineStr"/>
+      <c r="J53" s="16" t="inlineStr"/>
+      <c r="K53" s="17" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="4" t="inlineStr"/>
-      <c r="B54" s="4" t="inlineStr"/>
-      <c r="C54" s="4" t="inlineStr"/>
-      <c r="D54" s="4" t="inlineStr"/>
-      <c r="E54" s="4" t="inlineStr"/>
-      <c r="F54" s="4" t="inlineStr"/>
-      <c r="G54" s="4" t="inlineStr"/>
-      <c r="H54" s="4" t="inlineStr"/>
-      <c r="I54" s="4" t="inlineStr"/>
-      <c r="J54" s="4" t="inlineStr"/>
-      <c r="K54" s="4" t="inlineStr"/>
+      <c r="A54" s="16" t="inlineStr"/>
+      <c r="B54" s="17" t="inlineStr"/>
+      <c r="C54" s="17" t="inlineStr"/>
+      <c r="D54" s="17" t="inlineStr"/>
+      <c r="E54" s="17" t="inlineStr"/>
+      <c r="F54" s="17" t="inlineStr"/>
+      <c r="G54" s="17" t="inlineStr"/>
+      <c r="H54" s="17" t="inlineStr"/>
+      <c r="I54" s="16" t="inlineStr"/>
+      <c r="J54" s="16" t="inlineStr"/>
+      <c r="K54" s="17" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="4" t="inlineStr"/>
-      <c r="B55" s="4" t="inlineStr"/>
-      <c r="C55" s="4" t="inlineStr"/>
-      <c r="D55" s="4" t="inlineStr"/>
-      <c r="E55" s="4" t="inlineStr"/>
-      <c r="F55" s="4" t="inlineStr"/>
-      <c r="G55" s="4" t="inlineStr"/>
-      <c r="H55" s="4" t="inlineStr"/>
-      <c r="I55" s="4" t="inlineStr"/>
-      <c r="J55" s="4" t="inlineStr"/>
-      <c r="K55" s="4" t="inlineStr"/>
+      <c r="A55" s="16" t="inlineStr"/>
+      <c r="B55" s="17" t="inlineStr"/>
+      <c r="C55" s="17" t="inlineStr"/>
+      <c r="D55" s="17" t="inlineStr"/>
+      <c r="E55" s="17" t="inlineStr"/>
+      <c r="F55" s="17" t="inlineStr"/>
+      <c r="G55" s="17" t="inlineStr"/>
+      <c r="H55" s="17" t="inlineStr"/>
+      <c r="I55" s="16" t="inlineStr"/>
+      <c r="J55" s="16" t="inlineStr"/>
+      <c r="K55" s="17" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1538,18 +1607,45 @@
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A3:K3"/>
   </mergeCells>
-  <dataValidations count="4">
-    <dataValidation sqref="E6:E55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <conditionalFormatting sqref="A6:A55">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$A6="áno"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I6:I55">
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>$I6="odpísali"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="0">
+      <formula>$I6="stretnutie"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="1">
+      <formula>$I6="odmietli"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="2">
+      <formula>$I6="čakám na odpoveď"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C6:H55">
+    <cfRule type="expression" priority="6" dxfId="3">
+      <formula>$A6&lt;&gt;"áno"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="5">
+    <dataValidation sqref="A6:A55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"áno"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F6:F55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Re-RO,cez známeho,studené,inzerát"</formula1>
     </dataValidation>
-    <dataValidation sqref="F6:F55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G6:G55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"knižné,grafické"</formula1>
     </dataValidation>
-    <dataValidation sqref="H6:H55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"áno,nie,čaká sa"</formula1>
+    <dataValidation sqref="I6:I55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"čakám na odpoveď,odpísali,odmietli,stretnutie"</formula1>
     </dataValidation>
     <dataValidation sqref="J6:J55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"áno,nie"</formula1>
+      <formula1>"áno"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1562,7 +1658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1588,180 +1684,202 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Odoslaných spolu</t>
+          <t>Napísala som</t>
         </is>
       </c>
       <c r="B3" s="12">
-        <f>COUNTA(Oslovenia!A6:A55)</f>
+        <f>COUNTIF(Oslovenia!$A$6:$A$55,"áno")</f>
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Z toho odpovedalo</t>
+          <t>Odpísali</t>
         </is>
       </c>
       <c r="B4" s="12">
-        <f>COUNTIF(Oslovenia!H6:H55,"áno")</f>
+        <f>SUMPRODUCT((Oslovenia!$A$6:$A$55="áno")*((Oslovenia!$I$6:$I$55="odpísali")+(Oslovenia!$I$6:$I$55="stretnutie")))</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
+          <t>Odmietli</t>
+        </is>
+      </c>
+      <c r="B5" s="12">
+        <f>SUMPRODUCT((Oslovenia!$A$6:$A$55="áno")*(Oslovenia!$I$6:$I$55="odmietli"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Čakám na odpoveď</t>
+        </is>
+      </c>
+      <c r="B6" s="12">
+        <f>SUMPRODUCT((Oslovenia!$A$6:$A$55="áno")*(Oslovenia!$I$6:$I$55="čakám na odpoveď"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
           <t>Odpoveďovosť</t>
         </is>
       </c>
-      <c r="B5" s="8">
+      <c r="B7" s="8">
         <f>IFERROR(B4/B3,"")</f>
         <v/>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Podľa typu oslovenia</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>Typ</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Odoslané</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Odpovede</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>Napísala</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>Odpísali</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="inlineStr">
         <is>
           <t>Odpoveďovosť</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>Re-RO</t>
         </is>
       </c>
-      <c r="B9" s="13">
-        <f>SUMPRODUCT((Oslovenia!$E$6:$E$55=$A9)*(Oslovenia!$A$6:$A$55&lt;&gt;""))</f>
+      <c r="B11" s="20">
+        <f>SUMPRODUCT((Oslovenia!$F$6:$F$55=$A11)*(Oslovenia!$A$6:$A$55="áno"))</f>
         <v/>
       </c>
-      <c r="C9" s="13">
-        <f>SUMPRODUCT((Oslovenia!$E$6:$E$55=$A9)*(Oslovenia!$A$6:$A$55&lt;&gt;"")*(Oslovenia!$H$6:$H$55="áno"))</f>
+      <c r="C11" s="20">
+        <f>SUMPRODUCT((Oslovenia!$F$6:$F$55=$A11)*(Oslovenia!$A$6:$A$55="áno")*((Oslovenia!$I$6:$I$55="odpísali")+(Oslovenia!$I$6:$I$55="stretnutie")))</f>
         <v/>
       </c>
-      <c r="D9" s="9">
-        <f>IFERROR(C9/B9,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>cez známeho</t>
-        </is>
-      </c>
-      <c r="B10" s="13">
-        <f>SUMPRODUCT((Oslovenia!$E$6:$E$55=$A10)*(Oslovenia!$A$6:$A$55&lt;&gt;""))</f>
-        <v/>
-      </c>
-      <c r="C10" s="13">
-        <f>SUMPRODUCT((Oslovenia!$E$6:$E$55=$A10)*(Oslovenia!$A$6:$A$55&lt;&gt;"")*(Oslovenia!$H$6:$H$55="áno"))</f>
-        <v/>
-      </c>
-      <c r="D10" s="9">
-        <f>IFERROR(C10/B10,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>studené</t>
-        </is>
-      </c>
-      <c r="B11" s="13">
-        <f>SUMPRODUCT((Oslovenia!$E$6:$E$55=$A11)*(Oslovenia!$A$6:$A$55&lt;&gt;""))</f>
-        <v/>
-      </c>
-      <c r="C11" s="13">
-        <f>SUMPRODUCT((Oslovenia!$E$6:$E$55=$A11)*(Oslovenia!$A$6:$A$55&lt;&gt;"")*(Oslovenia!$H$6:$H$55="áno"))</f>
-        <v/>
-      </c>
-      <c r="D11" s="9">
+      <c r="D11" s="21">
         <f>IFERROR(C11/B11,"")</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>inzerát</t>
-        </is>
-      </c>
-      <c r="B12" s="13">
-        <f>SUMPRODUCT((Oslovenia!$E$6:$E$55=$A12)*(Oslovenia!$A$6:$A$55&lt;&gt;""))</f>
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>cez známeho</t>
+        </is>
+      </c>
+      <c r="B12" s="20">
+        <f>SUMPRODUCT((Oslovenia!$F$6:$F$55=$A12)*(Oslovenia!$A$6:$A$55="áno"))</f>
         <v/>
       </c>
-      <c r="C12" s="13">
-        <f>SUMPRODUCT((Oslovenia!$E$6:$E$55=$A12)*(Oslovenia!$A$6:$A$55&lt;&gt;"")*(Oslovenia!$H$6:$H$55="áno"))</f>
+      <c r="C12" s="20">
+        <f>SUMPRODUCT((Oslovenia!$F$6:$F$55=$A12)*(Oslovenia!$A$6:$A$55="áno")*((Oslovenia!$I$6:$I$55="odpísali")+(Oslovenia!$I$6:$I$55="stretnutie")))</f>
         <v/>
       </c>
-      <c r="D12" s="9">
+      <c r="D12" s="21">
         <f>IFERROR(C12/B12,"")</f>
         <v/>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>studené</t>
+        </is>
+      </c>
+      <c r="B13" s="20">
+        <f>SUMPRODUCT((Oslovenia!$F$6:$F$55=$A13)*(Oslovenia!$A$6:$A$55="áno"))</f>
+        <v/>
+      </c>
+      <c r="C13" s="20">
+        <f>SUMPRODUCT((Oslovenia!$F$6:$F$55=$A13)*(Oslovenia!$A$6:$A$55="áno")*((Oslovenia!$I$6:$I$55="odpísali")+(Oslovenia!$I$6:$I$55="stretnutie")))</f>
+        <v/>
+      </c>
+      <c r="D13" s="21">
+        <f>IFERROR(C13/B13,"")</f>
+        <v/>
+      </c>
+    </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>inzerát</t>
+        </is>
+      </c>
+      <c r="B14" s="20">
+        <f>SUMPRODUCT((Oslovenia!$F$6:$F$55=$A14)*(Oslovenia!$A$6:$A$55="áno"))</f>
+        <v/>
+      </c>
+      <c r="C14" s="20">
+        <f>SUMPRODUCT((Oslovenia!$F$6:$F$55=$A14)*(Oslovenia!$A$6:$A$55="áno")*((Oslovenia!$I$6:$I$55="odpísali")+(Oslovenia!$I$6:$I$55="stretnutie")))</f>
+        <v/>
+      </c>
+      <c r="D14" s="21">
+        <f>IFERROR(C14/B14,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Očakávané podľa knihy: Re-RO okolo 80 %, cez známeho vysoké, studené okolo 25 %. Ak si výrazne nižšie, chyba býva v tom, že pochvala nebola konkrétna.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>Metóda čiarok — cieľ 100 oslovení</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Metóda čiarok — cieľ 100</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>Hotovo</t>
         </is>
       </c>
-      <c r="B17" s="12">
-        <f>COUNTA(Oslovenia!A6:A55)</f>
+      <c r="B19" s="12">
+        <f>COUNTIF(Oslovenia!$A$6:$A$55,"áno")</f>
         <v/>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>Zostáva do stovky</t>
-        </is>
-      </c>
-      <c r="B18" s="12">
-        <f>MAX(0,100-B17)</f>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>Zostáva</t>
+        </is>
+      </c>
+      <c r="B20" s="12">
+        <f>MAX(0,100-B19)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="A16:D16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3354,6 +3472,11 @@
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
+  <conditionalFormatting sqref="F5:F26">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$F5="áno"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="F5:F26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"áno,nie"</formula1>
@@ -4384,6 +4507,11 @@
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
+  <conditionalFormatting sqref="D5:D57">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$D5="áno"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="D5:D57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"áno"</formula1>

</xml_diff>

<commit_message>
Apply to job ads the day they appear, not on Fridays
She pointed out two things the Friday rule ignored: a good ad is gone
within days, and the labour office requires documented proof that she
applied, which a batching rule delays. Both beat the tidiness the rule was
protecting.

Applications now happen the day she finds the ad, with a fifteen minute
check on each weekday. Friday keeps a slot, but as a catch-up for what
slipped and for filing the week's evidence. The cost of applying comes
down instead: a cover letter skeleton where only the first paragraph
changes, so a single application is ten minutes rather than an hour.

The ads sheet gains the link, how she applied, and where the proof is,
and the sheet now says to save each ad as a PDF at the moment of applying,
since it will not be on the web when the office asks about it.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CRJ8GE4B9NBudRKNSE36EN
</commit_message>
<xml_diff>
--- a/career/Viktoria-hladanie-prace.xlsx
+++ b/career/Viktoria-hladanie-prace.xlsx
@@ -116,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -161,6 +161,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3066,7 +3069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3076,6 +3079,9 @@
     <col width="42" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3085,10 +3091,10 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Stav k 27. 7. 2026, over si ich. Na inzerát sa hlásia desiatky ľudí a rozhoduje rýchlosť: posielaj naraz, nie po jednom. Prikladá sa CV a grafická verzia portfólia.</t>
+    <row r="2" ht="46" customHeight="1">
+      <c r="A2" s="22" t="inlineStr">
+        <is>
+          <t>Stav k 27. 7. 2026, over si ich. Na inzerát sa hlásia desiatky ľudí a rozhoduje rýchlosť: hláste sa v ten deň, keď inzerát nájdeš. Prikladá sa CV a portfólio. Inzerát si vždy ulož ako PDF hneď pri prihlásení, o mesiac už na webe nebude a bez neho nemáš čo doložiť úradu práce.</t>
         </is>
       </c>
     </row>
@@ -3126,6 +3132,21 @@
       <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Dátum</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Odkaz na inzerát</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Ako som sa prihlásila</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Doklad pre úrad práce</t>
         </is>
       </c>
     </row>
@@ -3469,8 +3490,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
   <conditionalFormatting sqref="F5:F26">
     <cfRule type="expression" priority="1" dxfId="0">

</xml_diff>

<commit_message>
Zapísať pohovory High5 a SNG do tabuľky
Oslovenia: dva riadky s výsledkom, odmietli a stretnutie.
Inzeráty: obe pozície s kanálom, cez ktorý sa prihlásila.
Úlohy: blok po pohovoroch, od ďakovného mailu po druhý kontakt
s High5 v novembri. Počítadlo hotových úloh a rozsah odškrtávania
posunuté na nové riadky.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CRJ8GE4B9NBudRKNSE36EN
</commit_message>
<xml_diff>
--- a/career/Viktoria-hladanie-prace.xlsx
+++ b/career/Viktoria-hladanie-prace.xlsx
@@ -1150,30 +1150,110 @@
       <c r="K20" s="17" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="16" t="inlineStr"/>
-      <c r="B21" s="17" t="inlineStr"/>
-      <c r="C21" s="17" t="inlineStr"/>
-      <c r="D21" s="17" t="inlineStr"/>
-      <c r="E21" s="17" t="inlineStr"/>
-      <c r="F21" s="17" t="inlineStr"/>
-      <c r="G21" s="17" t="inlineStr"/>
-      <c r="H21" s="17" t="inlineStr"/>
-      <c r="I21" s="16" t="inlineStr"/>
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>áno</t>
+        </is>
+      </c>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>doplniť</t>
+        </is>
+      </c>
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>kontakt z pohovoru</t>
+        </is>
+      </c>
+      <c r="D21" s="18" t="inlineStr">
+        <is>
+          <t>High5 — Mid/Senior Graphic Designer</t>
+        </is>
+      </c>
+      <c r="E21" s="18" t="inlineStr">
+        <is>
+          <t>doplniť</t>
+        </is>
+      </c>
+      <c r="F21" s="18" t="inlineStr">
+        <is>
+          <t>inzerát</t>
+        </is>
+      </c>
+      <c r="G21" s="18" t="inlineStr">
+        <is>
+          <t>grafické</t>
+        </is>
+      </c>
+      <c r="H21" s="17" t="inlineStr">
+        <is>
+          <t>Prihláška cez Pretlak</t>
+        </is>
+      </c>
+      <c r="I21" s="16" t="inlineStr">
+        <is>
+          <t>odmietli</t>
+        </is>
+      </c>
       <c r="J21" s="16" t="inlineStr"/>
-      <c r="K21" s="17" t="inlineStr"/>
+      <c r="K21" s="17" t="inlineStr">
+        <is>
+          <t>Pohovor absolvovaný. 18. 8. 2026 prišlo odmietnutie, vybrali kandidáta so skúsenosťami. V ten istý deň odpoveď s prosbou o jednu konkrétnu spätnú väzbu a s ponukou výpomoci, plus spojenie na LinkedIne. Ďalší kontakt november 2026 s jednou novou prácou.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="16" t="inlineStr"/>
-      <c r="B22" s="17" t="inlineStr"/>
-      <c r="C22" s="17" t="inlineStr"/>
-      <c r="D22" s="17" t="inlineStr"/>
-      <c r="E22" s="17" t="inlineStr"/>
-      <c r="F22" s="17" t="inlineStr"/>
-      <c r="G22" s="17" t="inlineStr"/>
-      <c r="H22" s="17" t="inlineStr"/>
-      <c r="I22" s="16" t="inlineStr"/>
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t>áno</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>doplniť</t>
+        </is>
+      </c>
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>Alexandra Pilo — HR manažérka</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>Slovenská národná galéria — junior grafik a DTP operátor</t>
+        </is>
+      </c>
+      <c r="E22" s="18" t="inlineStr">
+        <is>
+          <t>kariera@sng.sk, marta.kapustova@sng.sk</t>
+        </is>
+      </c>
+      <c r="F22" s="18" t="inlineStr">
+        <is>
+          <t>inzerát</t>
+        </is>
+      </c>
+      <c r="G22" s="18" t="inlineStr">
+        <is>
+          <t>grafické</t>
+        </is>
+      </c>
+      <c r="H22" s="17" t="inlineStr">
+        <is>
+          <t>Prihláška cez Profesiu a e-mailom</t>
+        </is>
+      </c>
+      <c r="I22" s="16" t="inlineStr">
+        <is>
+          <t>stretnutie</t>
+        </is>
+      </c>
       <c r="J22" s="16" t="inlineStr"/>
-      <c r="K22" s="17" t="inlineStr"/>
+      <c r="K22" s="17" t="inlineStr">
+        <is>
+          <t>Pohovor 17. 8. 2026 o 11:00, Riečna 1, viedla Alexandra Pilo. Mzda 1 400 až 1 600 € brutto podľa zákona 553/2003. Ďakovný mail do 24 hodín a spojenie na LinkedIne.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="16" t="inlineStr"/>
@@ -3354,22 +3434,98 @@
       <c r="G11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr"/>
-      <c r="B12" s="4" t="inlineStr"/>
-      <c r="C12" s="4" t="inlineStr"/>
-      <c r="D12" s="4" t="inlineStr"/>
-      <c r="E12" s="4" t="inlineStr"/>
-      <c r="F12" s="4" t="inlineStr"/>
-      <c r="G12" s="4" t="inlineStr"/>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Mid/Senior Graphic Designer</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>High5</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Bratislava</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>doplniť z inzerátu</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Agentúra, print aj online, ideamaking</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>áno</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>doplniť</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>pretlak.com</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Cez Pretlak</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr"/>
-      <c r="B13" s="4" t="inlineStr"/>
-      <c r="C13" s="4" t="inlineStr"/>
-      <c r="D13" s="4" t="inlineStr"/>
-      <c r="E13" s="4" t="inlineStr"/>
-      <c r="F13" s="4" t="inlineStr"/>
-      <c r="G13" s="4" t="inlineStr"/>
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Junior grafik a DTP operátor</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Slovenská národná galéria</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Bratislava</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>1 400 – 1 600 €</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>DTP a sadzba, navigačné systémy v priestore, tlačoviny k výstavám</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>áno</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>doplniť</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>profesia.sk</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Cez Profesiu a mail na kariera@sng.sk</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr"/>
@@ -3513,7 +3669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D59"/>
+  <dimension ref="A1:D67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4513,13 +4669,131 @@
       <c r="D57" s="4" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="C59" s="6" t="inlineStr">
-        <is>
-          <t>Hotových úloh z celkových 53</t>
-        </is>
-      </c>
-      <c r="D59" s="7">
-        <f>COUNTIF(D5:D57,"áno")</f>
+      <c r="A59" s="11" t="inlineStr"/>
+      <c r="B59" s="11" t="inlineStr"/>
+      <c r="C59" s="11" t="inlineStr">
+        <is>
+          <t>PO POHOVOROCH — august a november 2026</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="11" t="inlineStr">
+        <is>
+          <t>18. 8.</t>
+        </is>
+      </c>
+      <c r="B60" s="11" t="inlineStr">
+        <is>
+          <t>Utorok</t>
+        </is>
+      </c>
+      <c r="C60" s="11" t="inlineStr">
+        <is>
+          <t>SNG: ďakovný mail Alexandre Pilo. Do 24 hodín od pohovoru, teda dnes je posledný deň.</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="11" t="inlineStr">
+        <is>
+          <t>18. 8.</t>
+        </is>
+      </c>
+      <c r="B61" s="11" t="inlineStr">
+        <is>
+          <t>Utorok</t>
+        </is>
+      </c>
+      <c r="C61" s="11" t="inlineStr">
+        <is>
+          <t>SNG: žiadosť o spojenie na LinkedIne s Alexandrou Pilo, spolu s poďakovaním.</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="11" t="inlineStr">
+        <is>
+          <t>18. 8.</t>
+        </is>
+      </c>
+      <c r="B62" s="11" t="inlineStr">
+        <is>
+          <t>Utorok</t>
+        </is>
+      </c>
+      <c r="C62" s="11" t="inlineStr">
+        <is>
+          <t>High5: odpoveď na odmietnutie. Poďakovať, poprosiť o jednu konkrétnu spätnú väzbu, ponúknuť výpomoc.</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="11" t="inlineStr">
+        <is>
+          <t>18. 8.</t>
+        </is>
+      </c>
+      <c r="B63" s="11" t="inlineStr">
+        <is>
+          <t>Utorok</t>
+        </is>
+      </c>
+      <c r="C63" s="11" t="inlineStr">
+        <is>
+          <t>High5: žiadosť o spojenie na LinkedIne.</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="11" t="inlineStr">
+        <is>
+          <t>25. 8.</t>
+        </is>
+      </c>
+      <c r="B64" s="11" t="inlineStr">
+        <is>
+          <t>Utorok</t>
+        </is>
+      </c>
+      <c r="C64" s="11" t="inlineStr">
+        <is>
+          <t>SNG: ak sa do týždňa neozvú, jeden zdvorilý dotaz na stav výberového konania.</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="11" t="inlineStr">
+        <is>
+          <t>17. 11.</t>
+        </is>
+      </c>
+      <c r="B65" s="11" t="inlineStr">
+        <is>
+          <t>Pondelok</t>
+        </is>
+      </c>
+      <c r="C65" s="11" t="inlineStr">
+        <is>
+          <t>High5: druhý kontakt s jednou novou prácou. Nie prosba, len ukážka.</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="n"/>
+    </row>
+    <row r="67">
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Hotových úloh z celkových 59</t>
+        </is>
+      </c>
+      <c r="D67">
+        <f>COUNTIF(D5:D65,"áno")</f>
         <v/>
       </c>
     </row>
@@ -4534,7 +4808,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="D5:D57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D5:D65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"áno"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Doplnenie prehľadu oslovení a inzerátov do tabuľky
Do hárku Oslovenia pribudlo sedem riadkov s firmami, na ktoré Viktória
odpovedala na inzerát, do hárku Inzeráty stav prihlášok vrátane pohovoru
v SNG a odmietnutia z High5.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CRJ8GE4B9NBudRKNSE36EN
</commit_message>
<xml_diff>
--- a/career/Viktoria-hladanie-prace.xlsx
+++ b/career/Viktoria-hladanie-prace.xlsx
@@ -1162,12 +1162,12 @@
       </c>
       <c r="C21" s="18" t="inlineStr">
         <is>
-          <t>kontakt z pohovoru</t>
+          <t>doplniť</t>
         </is>
       </c>
       <c r="D21" s="18" t="inlineStr">
         <is>
-          <t>High5 — Mid/Senior Graphic Designer</t>
+          <t>Kempelenov inštitút inteligentných technológií — graphic designer</t>
         </is>
       </c>
       <c r="E21" s="18" t="inlineStr">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="H21" s="17" t="inlineStr">
         <is>
-          <t>Prihláška cez Pretlak</t>
+          <t>Prihláška cez Profesiu</t>
         </is>
       </c>
       <c r="I21" s="16" t="inlineStr">
@@ -1195,10 +1195,10 @@
           <t>odmietli</t>
         </is>
       </c>
-      <c r="J21" s="16" t="inlineStr"/>
+      <c r="J21" s="16" t="n"/>
       <c r="K21" s="17" t="inlineStr">
         <is>
-          <t>Pohovor absolvovaný. 18. 8. 2026 prišlo odmietnutie, vybrali kandidáta so skúsenosťami. V ten istý deň odpoveď s prosbou o jednu konkrétnu spätnú väzbu a s ponukou výpomoci, plus spojenie na LinkedIne. Ďalší kontakt november 2026 s jednou novou prácou.</t>
+          <t>Sky Park Offices, Bottova, Bratislava. 1 800 € mesačne, občas práca z domu.</t>
         </is>
       </c>
     </row>
@@ -1210,115 +1210,315 @@
       </c>
       <c r="B22" s="17" t="inlineStr">
         <is>
+          <t>utorok 4. 8. 2026 (over si)</t>
+        </is>
+      </c>
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>kontakt z pohovoru</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>High5 — Mid/Senior Graphic Designer</t>
+        </is>
+      </c>
+      <c r="E22" s="18" t="inlineStr">
+        <is>
           <t>doplniť</t>
         </is>
       </c>
-      <c r="C22" s="18" t="inlineStr">
+      <c r="F22" s="18" t="inlineStr">
+        <is>
+          <t>inzerát</t>
+        </is>
+      </c>
+      <c r="G22" s="18" t="inlineStr">
+        <is>
+          <t>grafické</t>
+        </is>
+      </c>
+      <c r="H22" s="17" t="inlineStr">
+        <is>
+          <t>Prihláška cez Pretlak</t>
+        </is>
+      </c>
+      <c r="I22" s="16" t="inlineStr">
+        <is>
+          <t>odmietli</t>
+        </is>
+      </c>
+      <c r="J22" s="16" t="n"/>
+      <c r="K22" s="17" t="inlineStr">
+        <is>
+          <t>Bratislava, od 1 800 €. Pohovor absolvovaný. 18. 8. 2026 odmietnutie, vybrali kandidáta so skúsenosťami. V ten deň odpoveď s prosbou o jednu konkrétnu spätnú väzbu a ponukou výpomoci, plus spojenie na LinkedIne. Druhý kontakt november 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>áno</t>
+        </is>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>utorok 4. 8. 2026 (over si)</t>
+        </is>
+      </c>
+      <c r="C23" s="18" t="inlineStr">
+        <is>
+          <t>doplniť</t>
+        </is>
+      </c>
+      <c r="D23" s="18" t="inlineStr">
+        <is>
+          <t>Expresta — externý grafik</t>
+        </is>
+      </c>
+      <c r="E23" s="18" t="inlineStr">
+        <is>
+          <t>doplniť</t>
+        </is>
+      </c>
+      <c r="F23" s="18" t="inlineStr">
+        <is>
+          <t>inzerát</t>
+        </is>
+      </c>
+      <c r="G23" s="18" t="inlineStr">
+        <is>
+          <t>grafické</t>
+        </is>
+      </c>
+      <c r="H23" s="17" t="inlineStr">
+        <is>
+          <t>Prihláška cez Profesiu</t>
+        </is>
+      </c>
+      <c r="I23" s="16" t="inlineStr">
+        <is>
+          <t>čakám na odpoveď</t>
+        </is>
+      </c>
+      <c r="J23" s="16" t="n"/>
+      <c r="K23" s="17" t="inlineStr">
+        <is>
+          <t>Bratislava, práca z domu, na živnosť, 500 až 2 500 €.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="16" t="inlineStr">
+        <is>
+          <t>áno</t>
+        </is>
+      </c>
+      <c r="B24" s="17" t="inlineStr">
+        <is>
+          <t>11. 8. 2026</t>
+        </is>
+      </c>
+      <c r="C24" s="18" t="inlineStr">
         <is>
           <t>Alexandra Pilo — HR manažérka</t>
         </is>
       </c>
-      <c r="D22" s="18" t="inlineStr">
+      <c r="D24" s="18" t="inlineStr">
         <is>
           <t>Slovenská národná galéria — junior grafik a DTP operátor</t>
         </is>
       </c>
-      <c r="E22" s="18" t="inlineStr">
+      <c r="E24" s="18" t="inlineStr">
         <is>
           <t>kariera@sng.sk, marta.kapustova@sng.sk</t>
         </is>
       </c>
-      <c r="F22" s="18" t="inlineStr">
+      <c r="F24" s="18" t="inlineStr">
         <is>
           <t>inzerát</t>
         </is>
       </c>
-      <c r="G22" s="18" t="inlineStr">
+      <c r="G24" s="18" t="inlineStr">
         <is>
           <t>grafické</t>
         </is>
       </c>
-      <c r="H22" s="17" t="inlineStr">
+      <c r="H24" s="17" t="inlineStr">
         <is>
           <t>Prihláška cez Profesiu a e-mailom</t>
         </is>
       </c>
-      <c r="I22" s="16" t="inlineStr">
+      <c r="I24" s="16" t="inlineStr">
         <is>
           <t>stretnutie</t>
         </is>
       </c>
-      <c r="J22" s="16" t="inlineStr"/>
-      <c r="K22" s="17" t="inlineStr">
-        <is>
-          <t>Pohovor 17. 8. 2026 o 11:00, Riečna 1, viedla Alexandra Pilo. Mzda 1 400 až 1 600 € brutto podľa zákona 553/2003. Ďakovný mail do 24 hodín a spojenie na LinkedIne.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="16" t="inlineStr"/>
-      <c r="B23" s="17" t="inlineStr"/>
-      <c r="C23" s="17" t="inlineStr"/>
-      <c r="D23" s="17" t="inlineStr"/>
-      <c r="E23" s="17" t="inlineStr"/>
-      <c r="F23" s="17" t="inlineStr"/>
-      <c r="G23" s="17" t="inlineStr"/>
-      <c r="H23" s="17" t="inlineStr"/>
-      <c r="I23" s="16" t="inlineStr"/>
-      <c r="J23" s="16" t="inlineStr"/>
-      <c r="K23" s="17" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="16" t="inlineStr"/>
-      <c r="B24" s="17" t="inlineStr"/>
-      <c r="C24" s="17" t="inlineStr"/>
-      <c r="D24" s="17" t="inlineStr"/>
-      <c r="E24" s="17" t="inlineStr"/>
-      <c r="F24" s="17" t="inlineStr"/>
-      <c r="G24" s="17" t="inlineStr"/>
-      <c r="H24" s="17" t="inlineStr"/>
-      <c r="I24" s="16" t="inlineStr"/>
-      <c r="J24" s="16" t="inlineStr"/>
-      <c r="K24" s="17" t="inlineStr"/>
+      <c r="J24" s="16" t="n"/>
+      <c r="K24" s="17" t="inlineStr">
+        <is>
+          <t>Pohovor 17. 8. 2026 o 11:00, Riečna 1, viedla Alexandra Pilo. 1 400 až 1 600 € brutto podľa zákona 553/2003. Ďakovný mail do 24 hodín a spojenie na LinkedIne.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="16" t="inlineStr"/>
-      <c r="B25" s="17" t="inlineStr"/>
-      <c r="C25" s="17" t="inlineStr"/>
-      <c r="D25" s="17" t="inlineStr"/>
-      <c r="E25" s="17" t="inlineStr"/>
-      <c r="F25" s="17" t="inlineStr"/>
-      <c r="G25" s="17" t="inlineStr"/>
-      <c r="H25" s="17" t="inlineStr"/>
-      <c r="I25" s="16" t="inlineStr"/>
-      <c r="J25" s="16" t="inlineStr"/>
-      <c r="K25" s="17" t="inlineStr"/>
+      <c r="A25" s="16" t="inlineStr">
+        <is>
+          <t>áno</t>
+        </is>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>11. 8. 2026</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="inlineStr">
+        <is>
+          <t>doplniť</t>
+        </is>
+      </c>
+      <c r="D25" s="18" t="inlineStr">
+        <is>
+          <t>FixDistribution s. r. o. — grafik / grafička</t>
+        </is>
+      </c>
+      <c r="E25" s="18" t="inlineStr">
+        <is>
+          <t>doplniť</t>
+        </is>
+      </c>
+      <c r="F25" s="18" t="inlineStr">
+        <is>
+          <t>inzerát</t>
+        </is>
+      </c>
+      <c r="G25" s="18" t="inlineStr">
+        <is>
+          <t>grafické</t>
+        </is>
+      </c>
+      <c r="H25" s="17" t="inlineStr">
+        <is>
+          <t>Prihláška cez Prácu za rohom</t>
+        </is>
+      </c>
+      <c r="I25" s="16" t="inlineStr">
+        <is>
+          <t>čakám na odpoveď</t>
+        </is>
+      </c>
+      <c r="J25" s="16" t="n"/>
+      <c r="K25" s="17" t="inlineStr">
+        <is>
+          <t>Odborárska, Bratislava. 1 500 až 1 800 € brutto, plný úväzok.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="16" t="inlineStr"/>
-      <c r="B26" s="17" t="inlineStr"/>
-      <c r="C26" s="17" t="inlineStr"/>
-      <c r="D26" s="17" t="inlineStr"/>
-      <c r="E26" s="17" t="inlineStr"/>
-      <c r="F26" s="17" t="inlineStr"/>
-      <c r="G26" s="17" t="inlineStr"/>
-      <c r="H26" s="17" t="inlineStr"/>
-      <c r="I26" s="16" t="inlineStr"/>
-      <c r="J26" s="16" t="inlineStr"/>
-      <c r="K26" s="17" t="inlineStr"/>
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t>áno</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>11. 8. 2026</t>
+        </is>
+      </c>
+      <c r="C26" s="18" t="inlineStr">
+        <is>
+          <t>doplniť</t>
+        </is>
+      </c>
+      <c r="D26" s="18" t="inlineStr">
+        <is>
+          <t>ŠEVT a. s. — grafik / grafička</t>
+        </is>
+      </c>
+      <c r="E26" s="18" t="inlineStr">
+        <is>
+          <t>doplniť</t>
+        </is>
+      </c>
+      <c r="F26" s="18" t="inlineStr">
+        <is>
+          <t>inzerát</t>
+        </is>
+      </c>
+      <c r="G26" s="18" t="inlineStr">
+        <is>
+          <t>grafické</t>
+        </is>
+      </c>
+      <c r="H26" s="17" t="inlineStr">
+        <is>
+          <t>Prihláška cez Prácu za rohom</t>
+        </is>
+      </c>
+      <c r="I26" s="16" t="inlineStr">
+        <is>
+          <t>čakám na odpoveď</t>
+        </is>
+      </c>
+      <c r="J26" s="16" t="n"/>
+      <c r="K26" s="17" t="inlineStr">
+        <is>
+          <t>Polus Tower 1, Vajnorská 100/A, Nové Mesto. Od 1 500 € brutto. Bez zaslaného portfólia žiadosť neakceptujú. Súčasťou výberu je zadanie.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="16" t="inlineStr"/>
-      <c r="B27" s="17" t="inlineStr"/>
-      <c r="C27" s="17" t="inlineStr"/>
-      <c r="D27" s="17" t="inlineStr"/>
-      <c r="E27" s="17" t="inlineStr"/>
-      <c r="F27" s="17" t="inlineStr"/>
-      <c r="G27" s="17" t="inlineStr"/>
-      <c r="H27" s="17" t="inlineStr"/>
-      <c r="I27" s="16" t="inlineStr"/>
-      <c r="J27" s="16" t="inlineStr"/>
-      <c r="K27" s="17" t="inlineStr"/>
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>áno</t>
+        </is>
+      </c>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>14. 8. 2026</t>
+        </is>
+      </c>
+      <c r="C27" s="18" t="inlineStr">
+        <is>
+          <t>doplniť</t>
+        </is>
+      </c>
+      <c r="D27" s="18" t="inlineStr">
+        <is>
+          <t>Wiktor Leo Burnett — graphic designer</t>
+        </is>
+      </c>
+      <c r="E27" s="18" t="inlineStr">
+        <is>
+          <t>doplniť</t>
+        </is>
+      </c>
+      <c r="F27" s="18" t="inlineStr">
+        <is>
+          <t>inzerát</t>
+        </is>
+      </c>
+      <c r="G27" s="18" t="inlineStr">
+        <is>
+          <t>grafické</t>
+        </is>
+      </c>
+      <c r="H27" s="17" t="inlineStr">
+        <is>
+          <t>Prihláška cez Pretlak</t>
+        </is>
+      </c>
+      <c r="I27" s="16" t="inlineStr">
+        <is>
+          <t>čakám na odpoveď</t>
+        </is>
+      </c>
+      <c r="J27" s="16" t="n"/>
+      <c r="K27" s="17" t="inlineStr">
+        <is>
+          <t>Bratislava, od 1 800 € na faktúru, teda treba živnosť. Mid seniorita, v požiadavkách 3 roky praxe v agentúre.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="16" t="inlineStr"/>
@@ -3314,8 +3514,26 @@
           <t>Bežná grafika, dobrá mzda</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr"/>
-      <c r="G7" s="4" t="inlineStr"/>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>áno</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>11. 8. 2026</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>pracazarohom.sk</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Cez Prácu za rohom</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -3340,11 +3558,29 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Publikácie a vizuály výskumného inštitútu</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr"/>
-      <c r="G8" s="4" t="inlineStr"/>
+          <t>Publikácie a vizuály výskumného inštitútu. Odmietnutie.</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>áno</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>doplniť</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>profesia.sk</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Cez Profesiu</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -3451,7 +3687,7 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>doplniť z inzerátu</t>
+          <t>od 1 800 €</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -3466,7 +3702,7 @@
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>doplniť</t>
+          <t>utorok 4. 8. 2026 (over si)</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -3513,7 +3749,7 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>doplniť</t>
+          <t>11. 8. 2026</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -3528,31 +3764,148 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr"/>
-      <c r="B14" s="4" t="inlineStr"/>
-      <c r="C14" s="4" t="inlineStr"/>
-      <c r="D14" s="4" t="inlineStr"/>
-      <c r="E14" s="4" t="inlineStr"/>
-      <c r="F14" s="4" t="inlineStr"/>
-      <c r="G14" s="4" t="inlineStr"/>
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Externý grafik</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Expresta</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Bratislava, práca z domu</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>500 – 2 500 €</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Príprava grafiky pre tlačoviny, na živnosť</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>áno</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>utorok 4. 8. 2026 (over si)</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>profesia.sk</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Cez Profesiu</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr"/>
-      <c r="B15" s="4" t="inlineStr"/>
-      <c r="C15" s="4" t="inlineStr"/>
-      <c r="D15" s="4" t="inlineStr"/>
-      <c r="E15" s="4" t="inlineStr"/>
-      <c r="F15" s="4" t="inlineStr"/>
-      <c r="G15" s="4" t="inlineStr"/>
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Grafik / grafička</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>ŠEVT a. s.</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Bratislava, Vajnorská 100/A</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>od 1 500 €</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Kontrola a príprava podkladov do tlače, print aj online</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>áno</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>11. 8. 2026</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>pracazarohom.sk</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Cez Prácu za rohom</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr"/>
-      <c r="B16" s="4" t="inlineStr"/>
-      <c r="C16" s="4" t="inlineStr"/>
-      <c r="D16" s="4" t="inlineStr"/>
-      <c r="E16" s="4" t="inlineStr"/>
-      <c r="F16" s="4" t="inlineStr"/>
-      <c r="G16" s="4" t="inlineStr"/>
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Graphic Designer</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Wiktor Leo Burnett</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Bratislava</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>od 1 800 €, faktúra</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Agentúra, print aj online, ideamaking</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>áno</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>14. 8. 2026</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>pretlak.com</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Cez Pretlak</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
Zapísať dve odoslané oslovenia
Riadok 16 dostal meno Ing. Patrik Jurkovič a funkciu hlavný majster
odbornej výchovy, riadok 17 pani Kardošovú. Obe s dátumom 18. 8.,
výsledok čakám na odpoveď a poznámkou o nudgi 25. 8.

Firma a funkcia pri riadku 17 ostáva doplniť, nevedel som ju overiť.
Prehľad sa prepočíta sám, jeho vzorce čítajú celý rozsah A6:A55.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CRJ8GE4B9NBudRKNSE36EN
</commit_message>
<xml_diff>
--- a/career/Viktoria-hladanie-prace.xlsx
+++ b/career/Viktoria-hladanie-prace.xlsx
@@ -1005,19 +1005,31 @@
       <c r="K15" s="17" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr"/>
-      <c r="B16" s="17" t="inlineStr"/>
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>áno</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>18. 8. 2026</t>
+        </is>
+      </c>
       <c r="C16" s="18" t="inlineStr">
         <is>
-          <t>[doplň meno]</t>
+          <t>Ing. Patrik Jurkovič</t>
         </is>
       </c>
       <c r="D16" s="18" t="inlineStr">
         <is>
-          <t>SOŠ polygrafická — učiteľ</t>
-        </is>
-      </c>
-      <c r="E16" s="18" t="n"/>
+          <t>SOŠ polygrafická — hlavný majster odbornej výchovy</t>
+        </is>
+      </c>
+      <c r="E16" s="18" t="inlineStr">
+        <is>
+          <t>doplniť</t>
+        </is>
+      </c>
       <c r="F16" s="18" t="inlineStr">
         <is>
           <t>Re-RO</t>
@@ -1028,25 +1040,49 @@
           <t>knižné</t>
         </is>
       </c>
-      <c r="H16" s="17" t="inlineStr"/>
-      <c r="I16" s="16" t="inlineStr"/>
+      <c r="H16" s="17" t="inlineStr">
+        <is>
+          <t>doplniť</t>
+        </is>
+      </c>
+      <c r="I16" s="16" t="inlineStr">
+        <is>
+          <t>čakám na odpoveď</t>
+        </is>
+      </c>
       <c r="J16" s="16" t="inlineStr"/>
-      <c r="K16" s="17" t="inlineStr"/>
+      <c r="K16" s="17" t="inlineStr">
+        <is>
+          <t>Nudge 25. 8., ak bude ticho</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr"/>
-      <c r="B17" s="17" t="inlineStr"/>
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>áno</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>18. 8. 2026</t>
+        </is>
+      </c>
       <c r="C17" s="18" t="inlineStr">
         <is>
-          <t>[doplň meno]</t>
+          <t>pani Kardošová</t>
         </is>
       </c>
       <c r="D17" s="18" t="inlineStr">
         <is>
-          <t>SOŠ polygrafická — učiteľ</t>
-        </is>
-      </c>
-      <c r="E17" s="18" t="n"/>
+          <t>doplniť</t>
+        </is>
+      </c>
+      <c r="E17" s="18" t="inlineStr">
+        <is>
+          <t>doplniť</t>
+        </is>
+      </c>
       <c r="F17" s="18" t="inlineStr">
         <is>
           <t>Re-RO</t>
@@ -1057,10 +1093,22 @@
           <t>knižné</t>
         </is>
       </c>
-      <c r="H17" s="17" t="inlineStr"/>
-      <c r="I17" s="16" t="inlineStr"/>
+      <c r="H17" s="17" t="inlineStr">
+        <is>
+          <t>doplniť</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>čakám na odpoveď</t>
+        </is>
+      </c>
       <c r="J17" s="16" t="inlineStr"/>
-      <c r="K17" s="17" t="inlineStr"/>
+      <c r="K17" s="17" t="inlineStr">
+        <is>
+          <t>Nudge 25. 8., ak bude ticho</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="16" t="inlineStr"/>
@@ -3809,7 +3857,6 @@
           <t>Cez Profesiu</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -3857,7 +3904,6 @@
           <t>Cez Prácu za rohom</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -3905,7 +3951,6 @@
           <t>Cez Pretlak</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
Doplniť inzeráty nájdené 18. 8.
Päť nových bratislavských pozícií do hárku Inzeráty, všetky so stavom
nie: KLARSTEIN, dm drogerie markt, MediaTech, Premedix a SLARA.

Riadky FaxCopy a Freshfields v tabuľke už boli od 27. júla. Overil som,
že oba inzeráty stále bežia, tak k nim pribudol odkaz a poznámka
o overení namiesto nových riadkov.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CRJ8GE4B9NBudRKNSE36EN
</commit_message>
<xml_diff>
--- a/career/Viktoria-hladanie-prace.xlsx
+++ b/career/Viktoria-hladanie-prace.xlsx
@@ -3501,11 +3501,16 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>DTP a príprava do tlače, presne tvoja priemyslovka</t>
+          <t>DTP a príprava do tlače, presne tvoja priemyslovka. Overené 18. 8., inzerát stále beží a v texte píšu, že nemusíš byť profík.</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr"/>
       <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>pracazarohom.sk/dl/jd/PROF-6a4718b0-822d-4a57-9545-17e78e63c442</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -3530,11 +3535,16 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Sadzba dlhých dokumentov v InDesigne, najlepšie platené</t>
+          <t>Sadzba dlhých dokumentov v InDesigne. Overené 18. 8., beží na ich vlastnom kariérnom webe. 4 dni práca, 4 dni voľno, 32 hodín týždenne.</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr"/>
       <c r="G6" s="4" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>freshfields.wd3.myworkdayjobs.com, pozícia R-06803-1</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -3953,67 +3963,212 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr"/>
-      <c r="B17" s="4" t="inlineStr"/>
-      <c r="C17" s="4" t="inlineStr"/>
-      <c r="D17" s="4" t="inlineStr"/>
-      <c r="E17" s="4" t="inlineStr"/>
-      <c r="F17" s="4" t="inlineStr"/>
-      <c r="G17" s="4" t="inlineStr"/>
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Motion &amp; Graphic Designer</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>KLARSTEIN (Berlin Brands Group)</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Bratislava, Grösslingová</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>od 1 600 €</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Motion, strih videa a AI nástroje. Nežiadajú počet rokov praxe.</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="n"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>profesia.sk/praca/klarstein-berlin-brands-group/O5331654</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr"/>
-      <c r="B18" s="4" t="inlineStr"/>
-      <c r="C18" s="4" t="inlineStr"/>
-      <c r="D18" s="4" t="inlineStr"/>
-      <c r="E18" s="4" t="inlineStr"/>
-      <c r="F18" s="4" t="inlineStr"/>
-      <c r="G18" s="4" t="inlineStr"/>
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Referent marketingu, obsah pre sociálne siete</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>dm drogerie markt</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Bratislava, Záhradnícka</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>2 196 €</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Presne to, čo robíš pre ShapelesAi. Najlepšie platené z celého zoznamu.</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="n"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>profesia.sk/praca/dm-drogerie-markt/O5335002</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr"/>
-      <c r="B19" s="4" t="inlineStr"/>
-      <c r="C19" s="4" t="inlineStr"/>
-      <c r="D19" s="4" t="inlineStr"/>
-      <c r="E19" s="4" t="inlineStr"/>
-      <c r="F19" s="4" t="inlineStr"/>
-      <c r="G19" s="4" t="inlineStr"/>
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Marketingový špecialista junior</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>MediaTech Central Europe</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Bratislava, Drieňová 34</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>od 1 500 €</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Junior pozícia, marketing s grafikou.</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="n"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>profesia.sk/praca/mediatech-central-europe/O5333256</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr"/>
-      <c r="B20" s="4" t="inlineStr"/>
-      <c r="C20" s="4" t="inlineStr"/>
-      <c r="D20" s="4" t="inlineStr"/>
-      <c r="E20" s="4" t="inlineStr"/>
-      <c r="F20" s="4" t="inlineStr"/>
-      <c r="G20" s="4" t="inlineStr"/>
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Graphic Designer</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Premedix</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Bratislava, Panenská 7</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>1 800 €</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Print aj digitál. Žiadajú 2 až 3 roky praxe, výber je na tri kolá so zadaním.</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="n"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>profesia.sk/praca/premedix/O5333707</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr"/>
-      <c r="B21" s="4" t="inlineStr"/>
-      <c r="C21" s="4" t="inlineStr"/>
-      <c r="D21" s="4" t="inlineStr"/>
-      <c r="E21" s="4" t="inlineStr"/>
-      <c r="F21" s="4" t="inlineStr"/>
-      <c r="G21" s="4" t="inlineStr"/>
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Grafik / kreatívny pracovník</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>SLARA</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Bratislava, Gagarinova</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>1 500 – 2 100 €</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Agentúra. Žiadajú 3 roky praxe a je to na živnosť. Bez portfólia CV nečítajú.</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>nie</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="n"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>profesia.sk/praca/slara/O3961268</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr"/>
-      <c r="B22" s="4" t="inlineStr"/>
-      <c r="C22" s="4" t="inlineStr"/>
-      <c r="D22" s="4" t="inlineStr"/>
-      <c r="E22" s="4" t="inlineStr"/>
-      <c r="F22" s="4" t="inlineStr"/>
-      <c r="G22" s="4" t="inlineStr"/>
+      <c r="A22" s="5" t="n"/>
+      <c r="B22" s="5" t="n"/>
+      <c r="C22" s="5" t="n"/>
+      <c r="D22" s="5" t="n"/>
+      <c r="E22" s="5" t="n"/>
+      <c r="F22" s="4" t="n"/>
+      <c r="G22" s="4" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr"/>
-      <c r="B23" s="4" t="inlineStr"/>
-      <c r="C23" s="4" t="inlineStr"/>
-      <c r="D23" s="4" t="inlineStr"/>
-      <c r="E23" s="4" t="inlineStr"/>
-      <c r="F23" s="4" t="inlineStr"/>
-      <c r="G23" s="4" t="inlineStr"/>
+      <c r="A23" s="5" t="n"/>
+      <c r="B23" s="5" t="n"/>
+      <c r="C23" s="5" t="n"/>
+      <c r="D23" s="5" t="n"/>
+      <c r="E23" s="5" t="n"/>
+      <c r="F23" s="4" t="n"/>
+      <c r="G23" s="4" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr"/>

</xml_diff>